<commit_message>
feat(frontend): update business workflows and simulator coverage
</commit_message>
<xml_diff>
--- a/docs/前后台联合测试执行记录-第十二轮-2026-09-28.xlsx
+++ b/docs/前后台联合测试执行记录-第十二轮-2026-09-28.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试总览" sheetId="1" r:id="Reb987d3c1291421e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试清单" sheetId="2" r:id="R22eb394cf05f40ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="准备与流程" sheetId="3" r:id="R57490809af9b450d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问题记录" sheetId="4" r:id="R23b4b45c82604cd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="自动手动组合" sheetId="5" r:id="R01aa153a8b9d4dfa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全流程验收" sheetId="6" r:id="Rba98c37e1dc14c5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="流程步骤记录" sheetId="7" r:id="R2cfbbcc7861a4182"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="审查结论" sheetId="8" r:id="R7d886d57a7aa4b46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="补充测试清单" sheetId="9" r:id="R8f70cb4191c74178"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设备运维清单" sheetId="10" r:id="R4311a5177f0d4d2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="本轮执行记录" sheetId="11" r:id="Reb519d27485d422a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试总览" sheetId="1" r:id="R3a65b74640a2461b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试清单" sheetId="2" r:id="Rbbab935eef1a4997"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="准备与流程" sheetId="3" r:id="Rb0e6064cd9254249"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问题记录" sheetId="4" r:id="Rd3922b663ae24df4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="自动手动组合" sheetId="5" r:id="R6a151a95af5a4cbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全流程验收" sheetId="6" r:id="R6f9388220af64d41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="流程步骤记录" sheetId="7" r:id="Rd6d9a72e5fc747b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="审查结论" sheetId="8" r:id="R42e80a4001af4156"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="补充测试清单" sheetId="9" r:id="R97f3469b870548dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设备运维清单" sheetId="10" r:id="Rd0521ed341544715"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="本轮执行记录" sheetId="11" r:id="R7c1232e57d514a95"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10656,7 +10656,7 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="328">
+  <x:cellXfs count="330">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -11621,6 +11621,12 @@
     <x:xf numFmtId="176" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="50">
     <x:cellStyle name="常规" xfId="0"/>
@@ -12461,7 +12467,7 @@
       </x:c>
       <x:c r="B6" s="254" t="n">
         <x:f>COUNTIF('测试清单'!$F$6:$F$157,"通过")</x:f>
-        <x:v>113</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="C6" s="255" t="n">
         <x:f>COUNTIF('测试清单'!$F$6:$F$157,"有问题")</x:f>
@@ -12469,7 +12475,7 @@
       </x:c>
       <x:c r="D6" s="256" t="n">
         <x:f>COUNTIF('测试清单'!$F$6:$F$157,"暂时测不了")</x:f>
-        <x:v>36</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="E6" s="257" t="n">
         <x:f>COUNTIF('测试清单'!$F$6:$F$157,"还没测")</x:f>
@@ -12481,7 +12487,7 @@
       </x:c>
       <x:c r="G6" s="259" t="n">
         <x:f>IF(A6-F6=0,"不适用",(B6+C6)/(A6-F6))</x:f>
-        <x:v>0.7583892617449665</x:v>
+        <x:v>0.8523489932885906</x:v>
       </x:c>
       <x:c r="H6" s="260" t="n">
         <x:f>IF(B6+C6=0,"尚未执行",B6/(B6+C6))</x:f>
@@ -12512,7 +12518,7 @@
     </x:row>
     <x:row r="9" ht="95" customHeight="1">
       <x:c r="A9" s="17" t="str">
-        <x:v>本轮新增49条完整条目通过；覆盖撤权、会话竞争、通知不可用与撤离停报、审批驳回、运维幂等、风险通知与并发冲突。</x:v>
+        <x:v>本轮新增63条完整条目通过；覆盖撤权、会话竞争、通知不可用与撤离停报、审批驳回、运维幂等、风险通知与并发冲突。</x:v>
       </x:c>
       <x:c r="B9" s="17"/>
       <x:c r="C9" s="17"/>
@@ -12524,7 +12530,7 @@
     </x:row>
     <x:row r="10" ht="95" customHeight="1">
       <x:c r="A10" s="17" t="str">
-        <x:v>完成44处代码修复，补齐计划状态测试入口；超视距评分配置仍待确认。短信3秒、电话10秒。</x:v>
+        <x:v>完成61处代码修复，补齐计划状态测试入口；超视距评分配置仍待确认。短信3秒、电话10秒。</x:v>
       </x:c>
       <x:c r="B10" s="17"/>
       <x:c r="C10" s="17"/>
@@ -12679,7 +12685,7 @@
       </x:c>
       <x:c r="C16" s="268" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A16,'测试清单'!$F$6:$F$157,"通过")</x:f>
-        <x:v>10</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D16" s="268" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A16,'测试清单'!$F$6:$F$157,"有问题")</x:f>
@@ -12687,7 +12693,7 @@
       </x:c>
       <x:c r="E16" s="268" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A16,'测试清单'!$F$6:$F$157,"暂时测不了")</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F16" s="268" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A16,'测试清单'!$F$6:$F$157,"还没测")</x:f>
@@ -12712,7 +12718,7 @@
       </x:c>
       <x:c r="C17" s="270" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A17,'测试清单'!$F$6:$F$157,"通过")</x:f>
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D17" s="270" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A17,'测试清单'!$F$6:$F$157,"有问题")</x:f>
@@ -12720,7 +12726,7 @@
       </x:c>
       <x:c r="E17" s="270" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A17,'测试清单'!$F$6:$F$157,"暂时测不了")</x:f>
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F17" s="270" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A17,'测试清单'!$F$6:$F$157,"还没测")</x:f>
@@ -12778,7 +12784,7 @@
       </x:c>
       <x:c r="C19" s="274" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A19,'测试清单'!$F$6:$F$157,"通过")</x:f>
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D19" s="274" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A19,'测试清单'!$F$6:$F$157,"有问题")</x:f>
@@ -12786,7 +12792,7 @@
       </x:c>
       <x:c r="E19" s="274" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A19,'测试清单'!$F$6:$F$157,"暂时测不了")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F19" s="274" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A19,'测试清单'!$F$6:$F$157,"还没测")</x:f>
@@ -12844,7 +12850,7 @@
       </x:c>
       <x:c r="C21" s="278" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A21,'测试清单'!$F$6:$F$157,"通过")</x:f>
-        <x:v>10</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D21" s="278" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A21,'测试清单'!$F$6:$F$157,"有问题")</x:f>
@@ -12852,7 +12858,7 @@
       </x:c>
       <x:c r="E21" s="278" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A21,'测试清单'!$F$6:$F$157,"暂时测不了")</x:f>
-        <x:v>8</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F21" s="278" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A21,'测试清单'!$F$6:$F$157,"还没测")</x:f>
@@ -12877,7 +12883,7 @@
       </x:c>
       <x:c r="C22" s="280" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A22,'测试清单'!$F$6:$F$157,"通过")</x:f>
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D22" s="280" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A22,'测试清单'!$F$6:$F$157,"有问题")</x:f>
@@ -12885,7 +12891,7 @@
       </x:c>
       <x:c r="E22" s="280" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A22,'测试清单'!$F$6:$F$157,"暂时测不了")</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F22" s="280" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A22,'测试清单'!$F$6:$F$157,"还没测")</x:f>
@@ -12943,7 +12949,7 @@
       </x:c>
       <x:c r="C24" s="284" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A24,'测试清单'!$F$6:$F$157,"通过")</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D24" s="284" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A24,'测试清单'!$F$6:$F$157,"有问题")</x:f>
@@ -12951,7 +12957,7 @@
       </x:c>
       <x:c r="E24" s="284" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A24,'测试清单'!$F$6:$F$157,"暂时测不了")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F24" s="284" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A24,'测试清单'!$F$6:$F$157,"还没测")</x:f>
@@ -13042,7 +13048,7 @@
       </x:c>
       <x:c r="C27" s="286" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A27,'测试清单'!$F$6:$F$157,"通过")</x:f>
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D27" s="286" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A27,'测试清单'!$F$6:$F$157,"有问题")</x:f>
@@ -13050,7 +13056,7 @@
       </x:c>
       <x:c r="E27" s="286" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A27,'测试清单'!$F$6:$F$157,"暂时测不了")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F27" s="286" t="n">
         <x:f>COUNTIFS('测试清单'!$B$6:$B$157,A27,'测试清单'!$F$6:$F$157,"还没测")</x:f>
@@ -13475,7 +13481,7 @@
       </x:c>
       <x:c r="H55" s="297" t="n">
         <x:f>COUNTIFS('测试清单'!F6:F157,"通过",'测试清单'!G6:G157,"&lt;&gt;",'测试清单'!H6:H157,"&lt;&gt;",'测试清单'!I6:I157,"&lt;&gt;",'测试清单'!J6:J157,"&lt;&gt;")+COUNTIFS('测试清单'!F6:F157,"不适用",'测试清单'!G6:G157,"&lt;&gt;")</x:f>
-        <x:v>116</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="16.5">
@@ -16667,7 +16673,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5155806411e04642"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46a6629dc88c41f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20571,16 +20577,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C195" s="310" t="str">
-        <x:v>主清单 68</x:v>
+        <x:v>主清单 11</x:v>
       </x:c>
       <x:c r="D195" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E195" s="310" t="str">
-        <x:v>短信配置过期时核实属实，短信BLOCKED、零通知记录，阶段AWAIT_COUNTER。续配后恢复发送作为后续独立状态保留。</x:v>
+        <x:v>两标签页各自会话不混用；甲退出后换乙、返回旧页可继续；网络拦截复现并修复甲迟到401清除乙新登录的缺陷。</x:v>
       </x:c>
       <x:c r="F195" s="310" t="str">
-        <x:v>qa-r12/sms-unavailable.json</x:v>
+        <x:v>qa-r12/race-fixed*.txt; two-tab-*.txt; auth-race-green.log</x:v>
       </x:c>
       <x:c r="G195" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -20594,16 +20600,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C196" s="310" t="str">
-        <x:v>主清单 69</x:v>
+        <x:v>主清单 16</x:v>
       </x:c>
       <x:c r="D196" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E196" s="310" t="str">
-        <x:v>实测短信送达后先WATCHING，3秒后因电话配置过期转待反制；原AUTO_CALL卡死已修复，电话零尝试、仅一条短信记录。</x:v>
+        <x:v>自然北京时间23:59:38今日45目标，00:00:09同页未刷新自动变1；MQTT跨日同一目标持续上报，44个前日停报目标被排除。API连续15秒采样同步验证，无改系统时间或业务库。</x:v>
       </x:c>
       <x:c r="F196" s="310" t="str">
-        <x:v>qa-r12/voice-unavailable.json; voice-unavailable-fixed.json; voice-unavailable-fixed.png; voice-phase-green-package.log</x:v>
+        <x:v>qa-r12/midnight-ui-2359.txt; midnight-ui-after.txt; midnight-ui-after.png; midnight-samples.json</x:v>
       </x:c>
       <x:c r="G196" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -20617,16 +20623,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C197" s="310" t="str">
-        <x:v>主清单 71</x:v>
+        <x:v>主清单 19</x:v>
       </x:c>
       <x:c r="D197" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E197" s="310" t="str">
-        <x:v>未核实及误报告警保持两渠道零尝试和零记录；开启模拟短信/电话后重复打开与刷新不触发通知。</x:v>
+        <x:v>正常MQTT双来源产生468个实测点，覆盖矩形转弯、末端298个停留位置点与33.365秒停报缺口；服务端缺口break_before=true，页面真实轨迹按段显示、不补缺失路线。独立停留目标返回同位置提示并保留灰色计划线。</x:v>
       </x:c>
       <x:c r="F197" s="310" t="str">
-        <x:v>qa-r12/unverified-false-positive-no-notification.json; no-notify-*.txt</x:v>
+        <x:v>qa-r12/trajectory-scene.json; trajectory-final.json; trajectory-gap-read.json; trajectory-red-green-grey-ui.png; trajectory-stationary-read.json; trajectory-stationary-ui.png</x:v>
       </x:c>
       <x:c r="G197" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -20640,16 +20646,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C198" s="310" t="str">
-        <x:v>主清单 11</x:v>
+        <x:v>主清单 20</x:v>
       </x:c>
       <x:c r="D198" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E198" s="310" t="str">
-        <x:v>两标签页各自会话不混用；甲退出后换乙、返回旧页可继续；网络拦截复现并修复甲迟到401清除乙新登录的缺陷。</x:v>
+        <x:v>执行中计划正常MQTT实测点经PostGIS返回WITHIN/OUTSIDE，页面分别绿色/红色，未飞计划线保持灰色。独立轨迹证据页没有匹配航线依据时显示黄色关系未知及明确说明；后端缺航线与缺间隔回归通过，不用未知数据染成符合。</x:v>
       </x:c>
       <x:c r="F198" s="310" t="str">
-        <x:v>qa-r12/race-fixed*.txt; two-tab-*.txt; auth-race-green.log</x:v>
+        <x:v>qa-r12/trajectory-final.json; trajectory-red-green-grey-ui.png; same-name-evidence-b-loaded.txt; same-name-evidence-b.png; rule-param-green.log</x:v>
       </x:c>
       <x:c r="G198" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -20663,16 +20669,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C199" s="310" t="str">
-        <x:v>主清单 64</x:v>
+        <x:v>主清单 21</x:v>
       </x:c>
       <x:c r="D199" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E199" s="310" t="str">
-        <x:v>只读账号无核实入口且服务端403；有操作权限但当前依据不足时明确阻止反制。</x:v>
+        <x:v>态势页真实本地HLS播放后收起video=0，切目标038清除旧039画面，离页释放；无任务明确说明，真实只读账号UI无权限且API403，测试画面标识保留。</x:v>
       </x:c>
       <x:c r="F199" s="310" t="str">
-        <x:v>qa-r12/readonly-alarm.txt; readonly-verify-denied.json; drop-counter-blocked.png</x:v>
+        <x:v>qa-r12/video-r18/situation-playing.png; situation-switched.txt; reader-situation-no-permission.txt; reader-video-permission.json</x:v>
       </x:c>
       <x:c r="G199" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -20686,16 +20692,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C200" s="310" t="str">
-        <x:v>主清单 72</x:v>
+        <x:v>主清单 26</x:v>
       </x:c>
       <x:c r="D200" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E200" s="310" t="str">
-        <x:v>短信后目标停报、设备心跳持续；修复预测轨迹被当新观测后，仅短信一条、电话BLOCKED零拨号、观察UNKNOWN，反制被明确阻止。</x:v>
+        <x:v>独立PostgreSQL/PostGIS同一到时执行计划未匹配目标：正常GOOD显示疑似未按计划起飞；BAD显示设备异常、是否起飞待确认；UNKNOWN显示信息不完整。真实前台三分支与API结论一致，不以无目标认定未起飞。</x:v>
       </x:c>
       <x:c r="F200" s="310" t="str">
-        <x:v>qa-r12/drop-sms-fixed.json; drop-counter-blocked.png; prediction-departure-green-package.log</x:v>
+        <x:v>qa-r12/maintenance-browser/postgres-fifth/normal-api.json；maintenance-browser/postgres-fifth/normal-ui.txt；maintenance-browser/postgres-fifth/unknown-api.json；maintenance-browser/postgres-fifth/unknown-ui.txt；maintenance-browser/postgres-fifth/abnormal-api.json；maintenance-browser/postgres-fifth/abnormal-ui.txt；due-plan-matrix-fixed-preflight.log</x:v>
       </x:c>
       <x:c r="G200" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -20709,16 +20715,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C201" s="310" t="str">
-        <x:v>主清单 81</x:v>
+        <x:v>主清单 28</x:v>
       </x:c>
       <x:c r="D201" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E201" s="310" t="str">
-        <x:v>实际页面驳回曾500，追加迁移010修复后原表单成功；另一有权账号批准200，申请人自批409，旧版本重批409。实际审批人及时间保存、驳回无有效期。</x:v>
+        <x:v>页面通知模拟离线设备，实际产生一张待办和一条模拟送达/签收；同异常同幂等键与不同幂等键并发三次均复用同任务，通知尝试保持1。</x:v>
       </x:c>
       <x:c r="F201" s="310" t="str">
-        <x:v>qa-r12/approval-rejection-cancellation.json; rejection-fixed.png; rejection-green-package.log</x:v>
+        <x:v>qa-r12/maintenance-duplicate.json; maintenance-ui-result.json; maintenance-ui.txt</x:v>
       </x:c>
       <x:c r="G201" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -20732,16 +20738,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C202" s="310" t="str">
-        <x:v>主清单 28</x:v>
+        <x:v>主清单 29</x:v>
       </x:c>
       <x:c r="D202" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E202" s="310" t="str">
-        <x:v>页面通知模拟离线设备，实际产生一张待办和一条模拟送达/签收；同异常同幂等键与不同幂等键并发三次均复用同任务，通知尝试保持1。</x:v>
+        <x:v>完全覆盖、部分覆盖、无覆盖已使用正常API计划和预报在浏览器验证。缺时间作为防御分支，以CDP只改一次详情响应start_at/end_at为null，实际天气接口保持真实；页面显示计划飞行时段不完整/无法确定对应预报时段，不展示任意时段。后台计划前后完全一致，拦截清除并重载真实页面。</x:v>
       </x:c>
       <x:c r="F202" s="310" t="str">
-        <x:v>qa-r12/maintenance-duplicate.json; maintenance-ui-result.json; maintenance-ui.txt</x:v>
+        <x:v>qa-r12/weather-full.txt; weather-partial.txt; weather-none.txt; weather-coverage-plans.json; weather-missing-time-source.json; weather-missing-time-ui.txt; weather-missing-time.png</x:v>
       </x:c>
       <x:c r="G202" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -20755,16 +20761,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C203" s="310" t="str">
-        <x:v>主清单 52</x:v>
+        <x:v>主清单 32</x:v>
       </x:c>
       <x:c r="D203" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E203" s="310" t="str">
-        <x:v>管理员从风险页面提交上级模拟通知，DELIVERED与PENDING签收分别显示；只读账号403，已修正误启用按钮。历史回放风险不代表当前持续风险。</x:v>
+        <x:v>同名A/B详情与天气延迟响应不串页；新建同名执行中计划、完成及取消计划，逐一核对身份和当前规则显示。修复计划+目标跳转时清空计划筛选及跨计划读取最新研判；两份计划分别进入各自目标与轨迹证据，B完整加载496点，5项回归通过。</x:v>
       </x:c>
       <x:c r="F203" s="310" t="str">
-        <x:v>qa-r12/risk-notification-success.txt; risk-notification-api.json</x:v>
+        <x:v>qa-r12/same-name-late-detail.txt; same-name-late-weather.png; state-plans.json; completed-plan-ui.txt; cancelled-plan-ui.txt; legality-plan-filter-fixed.txt; same-name-legality-b.txt; same-name-evidence-a.txt; same-name-evidence-b-loaded.txt; same-name-plan-filter-fixed.png</x:v>
       </x:c>
       <x:c r="G203" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -20778,16 +20784,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C204" s="310" t="str">
-        <x:v>主清单 134</x:v>
+        <x:v>主清单 35</x:v>
       </x:c>
       <x:c r="D204" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E204" s="310" t="str">
-        <x:v>四策略已分别验证：短信撤离LEFT且无电话、电话后10秒LEFT、持续飞行待反制、短信停报UNKNOWN且不拨号；全部MOCK/replay，无真实通知。</x:v>
+        <x:v>补齐仅研判可读而告警不可读账号：核实位置告警页面叠加非法仍显示1条，合法性页面叠加非法0条；详情保留并入既有告警事实，前往告警禁用且告警API403，不把无查看权限当无关联。角色已恢复。</x:v>
       </x:c>
       <x:c r="F204" s="310" t="str">
-        <x:v>qa-r12/sms-departure-fixed.json; voice-departure-fixed.json; drop-sms-fixed.json</x:v>
+        <x:v>qa-r12/legality-no-alarm-permission-api.json; legality-no-alarm-permission-ui.txt; legality-no-alarm-permission-ui.png; reader-role-restored-final.json</x:v>
       </x:c>
       <x:c r="G204" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -20801,16 +20807,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C205" s="310" t="str">
-        <x:v>主清单 141</x:v>
+        <x:v>主清单 40</x:v>
       </x:c>
       <x:c r="D205" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E205" s="310" t="str">
-        <x:v>两个独立人员会话并发核实、审批与撤销，均一方成功、另一方409版本冲突；旧审批页提交后自动回读已撤销，无覆盖。</x:v>
+        <x:v>既有CONFIRMED/REJECTED/OVERRIDDEN服务端和页面筛选已核对。本轮正常回放观测形成21条SUFFICIENT、review_required=false、review PENDING_REVIEW/version0记录；固定15秒窗口未复核记录3条，needs_review=true为0，false为3。页面非法21条切待复核为0，未把所有从未人工操作的记录归入待复核。DEMO参数警示保留；仅验筛选逻辑，不代表参数或算法准确性验收。</x:v>
       </x:c>
       <x:c r="F205" s="310" t="str">
-        <x:v>qa-r12/concurrent-verification.json; approval-cancel-race.json; stale-approval-cancelled.txt</x:v>
+        <x:v>qa-r12/review-state-transitions.json; review-filter-api.json; review-needs-latest.json; review-filter-confirmed.txt; review-filter-rejected.txt; review-filter-overridden.txt; review-not-required-positive.json; review-not-required-detail.json; review-not-required-before.txt; review-not-required-filtered.txt</x:v>
       </x:c>
       <x:c r="G205" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -20824,16 +20830,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C206" s="310" t="str">
-        <x:v>主清单 16</x:v>
+        <x:v>主清单 44</x:v>
       </x:c>
       <x:c r="D206" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E206" s="310" t="str">
-        <x:v>自然北京时间23:59:38今日45目标，00:00:09同页未刷新自动变1；MQTT跨日同一目标持续上报，44个前日停报目标被排除。API连续15秒采样同步验证，无改系统时间或业务库。</x:v>
+        <x:v>已通过正常分类修订API将独立QA无人机改判BIRD，原无人机深链清空详情且UAV列表不再包含该目标；另在浏览器精准阻断关联告警GET，页面明确网络失败，无核实入口，返回研判仍保留并入既有告警与前往告警入口，不按无告警放开重复复核。故障注入已解除。</x:v>
       </x:c>
       <x:c r="F206" s="310" t="str">
-        <x:v>qa-r12/midnight-ui-2359.txt; midnight-ui-after.txt; midnight-ui-after.png; midnight-samples.json</x:v>
+        <x:v>qa-r12/classification-change.json; classification-uav-before.txt; classification-non-uav-after.txt; associated-alarm-read-failed-ui.txt; associated-alarm-return-legality-ui.txt; associated-alarm-return-more-ui.txt</x:v>
       </x:c>
       <x:c r="G206" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -20847,16 +20853,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C207" s="310" t="str">
-        <x:v>主清单 35</x:v>
+        <x:v>主清单 48</x:v>
       </x:c>
       <x:c r="D207" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E207" s="310" t="str">
-        <x:v>补齐仅研判可读而告警不可读账号：核实位置告警页面叠加非法仍显示1条，合法性页面叠加非法0条；详情保留并入既有告警事实，前往告警禁用且告警API403，不把无查看权限当无关联。角色已恢复。</x:v>
+        <x:v>正常API发起039目标光电跟踪，实际MQTT BeginTracking回包，设备/目标/任务吻合；命令成功、TRACKING与HLS可用分别验证，960x540视频实际播放；结束MQTT回执后ENDED及旧HLS404。仅本地模拟验收。</x:v>
       </x:c>
       <x:c r="F207" s="310" t="str">
-        <x:v>qa-r12/legality-no-alarm-permission-api.json; legality-no-alarm-permission-ui.txt; legality-no-alarm-permission-ui.png; reader-role-restored-final.json</x:v>
+        <x:v>qa-r12/video-r18/business-started.json; business-player-proof.json; business-fixed-video.json; business-final.json; cleanup.json</x:v>
       </x:c>
       <x:c r="G207" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -20870,16 +20876,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C208" s="310" t="str">
-        <x:v>主清单 138</x:v>
+        <x:v>主清单 52</x:v>
       </x:c>
       <x:c r="D208" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E208" s="310" t="str">
-        <x:v>失效会话401回登录、无权限403明确拒绝、不存在计划404显示不存在、单请求500显示内部错误、实际15秒超时408分别核实；清除测试拦截后正常读取37条研判，不把异常当暂无数据。</x:v>
+        <x:v>管理员从风险页面提交上级模拟通知，DELIVERED与PENDING签收分别显示；只读账号403，已修正误启用按钮。历史回放风险不代表当前持续风险。</x:v>
       </x:c>
       <x:c r="F208" s="310" t="str">
-        <x:v>qa-r12/permission-revocation.json; legality-no-alarm-permission-api.json; ui-error-404.txt; ui-error-500.txt; ui-error-timeout.txt; ui-error-recovered.txt; ui-fault-test-summary.json</x:v>
+        <x:v>qa-r12/risk-notification-success.txt; risk-notification-api.json</x:v>
       </x:c>
       <x:c r="G208" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -20893,16 +20899,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C209" s="310" t="str">
-        <x:v>主清单 93</x:v>
+        <x:v>主清单 54</x:v>
       </x:c>
       <x:c r="D209" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E209" s="310" t="str">
-        <x:v>设备通道授权0009批准后、执行前撤销；刷新/重开仍已撤销无执行入口。上一轮真实协议急停0005重开并刷新仍反制已中止、allowed_actions为空，未恢复命令或授权。</x:v>
+        <x:v>补齐两条关联计划的真实 MQTT 鸟群风险，经 C04 规则计算、人工核验及模拟通道绑定，分别验证 SUBMITTED/PENDING、FAILED/NOT_EXPECTED、SUBMITTED/TIMEOUT、迟到 DELIVERED/PENDING 和 ACKNOWLEDGED；页面与接口一致。修复风险 NOTIFIED 误标已通知，改为通知已提交；失败显示尚未进入回执阶段。</x:v>
       </x:c>
       <x:c r="F209" s="310" t="str">
-        <x:v>qa-r12/approval-rejection-cancellation.json; stopped-task-reopened.txt; stopped-task-refreshed.txt; cancelled-task-reopened.txt; stop-cancel-final-state.json</x:v>
+        <x:v>qa-r12/risk-receipt-sequence.json; risk-timeout-fixed-ui.png; risk-failed-fixed-ui.txt; risk-delivered-ui.txt; risk-ack-ui.png</x:v>
       </x:c>
       <x:c r="G209" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -20916,16 +20922,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C210" s="310" t="str">
-        <x:v>主清单 137</x:v>
+        <x:v>主清单 56</x:v>
       </x:c>
       <x:c r="D210" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E210" s="310" t="str">
-        <x:v>页面暂停8秒发送计数和模拟进度不变，继续后增长；停止批次STOPPED。真实进程重启复现并修复中文批次丢失及进度未落盘；重启保留47秒136条且不续发。纯MQTT撤权后继续发送缺陷修复后约2秒自动停在58条；重新登录不自动恢复。</x:v>
+        <x:v>通过受限本地QA入口新增纯气象风险，实际时钟自然到期后CURRENT→UNKNOWN，核验/通知历史及版本不变；已过期天气和缺少新观测的鸟群风险均显示待确认，不视为解除。未来预警到时前不计当前。</x:v>
       </x:c>
       <x:c r="F210" s="310" t="str">
-        <x:v>qa-r12/simulator-control-samples.json; simulator-restart-fixed.png; simulator-session-expired-fixed.png; runtime-recovery-green-utf8.log; runtime-recovery-green-ansi.log; simulator-all-tests-final.log</x:v>
+        <x:v>qa-r12/weather-risk-natural-expiry.json; weather-risk-three-boundaries.json; weather-vs-nonweather-current.json; weather-current-plan-expired.txt; weather-risk-package-final.log</x:v>
       </x:c>
       <x:c r="G210" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -20939,16 +20945,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C211" s="310" t="str">
-        <x:v>主清单 100</x:v>
+        <x:v>主清单 64</x:v>
       </x:c>
       <x:c r="D211" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E211" s="310" t="str">
-        <x:v>同一真实模拟交接依次验证待发送、送达待确认、发送失败、已送达；原3次尝试分别保留PENDING_DELIVERY、FAILED、DELIVERED，页面查询不发送，未知不能算成功。</x:v>
+        <x:v>只读账号无核实入口且服务端403；有操作权限但当前依据不足时明确阻止反制。</x:v>
       </x:c>
       <x:c r="F211" s="310" t="str">
-        <x:v>qa-r12/handoff-pending-ui.txt; handoff-submitted-ui.txt; handoff-failed-ui.txt; handoff-delivered-timeout-ui.txt; handoff-receipt-invariants.json</x:v>
+        <x:v>qa-r12/readonly-alarm.txt; readonly-verify-denied.json; drop-counter-blocked.png</x:v>
       </x:c>
       <x:c r="G211" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -20962,16 +20968,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C212" s="310" t="str">
-        <x:v>主清单 101</x:v>
+        <x:v>主清单 65</x:v>
       </x:c>
       <x:c r="D212" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E212" s="310" t="str">
-        <x:v>未进入签收、等待签收、回执超时及已签收分别验证；迟到送达后保留送达时间，签收超时不抹掉送达。最终已签收但页面仍显示暂无关联案件结果，不认定处罚完成。</x:v>
+        <x:v>告警与反制详情默认展开实际测试HLS，收起video=0再展开；无任务、真实无权限、单次503分别提示；查看前后授权REQUESTED/version0一致，不触发反制。</x:v>
       </x:c>
       <x:c r="F212" s="310" t="str">
-        <x:v>qa-r12/handoff-receipt-sequence.json; handoff-timeout-ui.txt; handoff-delivered-timeout-ui.txt; handoff-acknowledged-ui.txt</x:v>
+        <x:v>qa-r12/video-r18/alarm-default-expanded.txt; authorization-video-expanded.txt; authorization-video-failed.txt; reader-authorization-no-permission.txt; authorization-before-view.json; authorization-after-view.json</x:v>
       </x:c>
       <x:c r="G212" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -20985,16 +20991,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C213" s="310" t="str">
-        <x:v>主清单 103</x:v>
+        <x:v>主清单 68</x:v>
       </x:c>
       <x:c r="D213" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E213" s="310" t="str">
-        <x:v>旧投递的迟到回执409，当前投递迟到送达可接受；成功不能回退失败409。重复签收同版本4重放不增长，夹带另一交接ID不改变真实关联，另一记录不变。</x:v>
+        <x:v>短信配置过期时核实属实，短信BLOCKED、零通知记录，阶段AWAIT_COUNTER。续配后恢复发送作为后续独立状态保留。</x:v>
       </x:c>
       <x:c r="F213" s="310" t="str">
-        <x:v>qa-r12/handoff-receipt-sequence.json; handoff-receipt-invariants.json</x:v>
+        <x:v>qa-r12/sms-unavailable.json</x:v>
       </x:c>
       <x:c r="G213" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21008,16 +21014,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C214" s="310" t="str">
-        <x:v>主清单 54</x:v>
+        <x:v>主清单 69</x:v>
       </x:c>
       <x:c r="D214" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E214" s="310" t="str">
-        <x:v>补齐两条关联计划的真实 MQTT 鸟群风险，经 C04 规则计算、人工核验及模拟通道绑定，分别验证 SUBMITTED/PENDING、FAILED/NOT_EXPECTED、SUBMITTED/TIMEOUT、迟到 DELIVERED/PENDING 和 ACKNOWLEDGED；页面与接口一致。修复风险 NOTIFIED 误标已通知，改为通知已提交；失败显示尚未进入回执阶段。</x:v>
+        <x:v>实测短信送达后先WATCHING，3秒后因电话配置过期转待反制；原AUTO_CALL卡死已修复，电话零尝试、仅一条短信记录。</x:v>
       </x:c>
       <x:c r="F214" s="310" t="str">
-        <x:v>qa-r12/risk-receipt-sequence.json; risk-timeout-fixed-ui.png; risk-failed-fixed-ui.txt; risk-delivered-ui.txt; risk-ack-ui.png</x:v>
+        <x:v>qa-r12/voice-unavailable.json; voice-unavailable-fixed.json; voice-unavailable-fixed.png; voice-phase-green-package.log</x:v>
       </x:c>
       <x:c r="G214" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21031,16 +21037,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C215" s="310" t="str">
-        <x:v>主清单 124</x:v>
+        <x:v>主清单 71</x:v>
       </x:c>
       <x:c r="D215" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E215" s="310" t="str">
-        <x:v>真实 MQTT workState=2→1，设备异常→在线，页面同一选中设备自动更新；整体健康仍UNKNOWN。当前测试页以浏览器媒体仿真启用prefers-reduced-motion，实际绘图函数常量静态红光22.5；普通模式6/17/28变化，恢复后不再应用红光。未改操作系统设置，测试后媒体仿真已撤销。</x:v>
+        <x:v>未核实及误报告警保持两渠道零尝试和零记录；开启模拟短信/电话后重复打开与刷新不触发通知。</x:v>
       </x:c>
       <x:c r="F215" s="310" t="str">
-        <x:v>qa-r12/motion-fault-api.json; motion-restored-api.json; motion-fault-ui.png; motion-restored-ui.png; motion-media-state.json; motion-function-verification.json</x:v>
+        <x:v>qa-r12/unverified-false-positive-no-notification.json; no-notify-*.txt</x:v>
       </x:c>
       <x:c r="G215" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21054,16 +21060,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C216" s="310" t="str">
-        <x:v>主清单 19</x:v>
+        <x:v>主清单 72</x:v>
       </x:c>
       <x:c r="D216" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E216" s="310" t="str">
-        <x:v>正常MQTT双来源产生468个实测点，覆盖矩形转弯、末端298个停留位置点与33.365秒停报缺口；服务端缺口break_before=true，页面真实轨迹按段显示、不补缺失路线。独立停留目标返回同位置提示并保留灰色计划线。</x:v>
+        <x:v>短信后目标停报、设备心跳持续；修复预测轨迹被当新观测后，仅短信一条、电话BLOCKED零拨号、观察UNKNOWN，反制被明确阻止。</x:v>
       </x:c>
       <x:c r="F216" s="310" t="str">
-        <x:v>qa-r12/trajectory-scene.json; trajectory-final.json; trajectory-gap-read.json; trajectory-red-green-grey-ui.png; trajectory-stationary-read.json; trajectory-stationary-ui.png</x:v>
+        <x:v>qa-r12/drop-sms-fixed.json; drop-counter-blocked.png; prediction-departure-green-package.log</x:v>
       </x:c>
       <x:c r="G216" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21077,16 +21083,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C217" s="310" t="str">
-        <x:v>主清单 32</x:v>
+        <x:v>主清单 74</x:v>
       </x:c>
       <x:c r="D217" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E217" s="310" t="str">
-        <x:v>同名A/B详情与天气延迟响应不串页；新建同名执行中计划、完成及取消计划，逐一核对身份和当前规则显示。修复计划+目标跳转时清空计划筛选及跨计划读取最新研判；两份计划分别进入各自目标与轨迹证据，B完整加载496点，5项回归通过。</x:v>
+        <x:v>补齐仅 local+qa / mock-replay / 精确事件生效的异常模拟入口；SENT 短信保持 UNKNOWN、0送达记录；NO_ANSWER 与 ANSWERED 未播完均 UNKNOWN、各1次，不写播放完成时间、不启动播放后观察、不显示反制入口。浏览器与正常API均核对。</x:v>
       </x:c>
       <x:c r="F217" s="310" t="str">
-        <x:v>qa-r12/same-name-late-detail.txt; same-name-late-weather.png; state-plans.json; completed-plan-ui.txt; cancelled-plan-ui.txt; legality-plan-filter-fixed.txt; same-name-legality-b.txt; same-name-evidence-a.txt; same-name-evidence-b-loaded.txt; same-name-plan-filter-fixed.png</x:v>
+        <x:v>qa-r12/advisory-sent-result.json；advisory-noanswer-result.json；advisory-noanswer-ui.txt；advisory-answered-phase-fixed.json；advisory-answered-fixed-expanded-ui.txt</x:v>
       </x:c>
       <x:c r="G217" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21100,16 +21106,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C218" s="310" t="str">
-        <x:v>主清单 20</x:v>
+        <x:v>主清单 79</x:v>
       </x:c>
       <x:c r="D218" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E218" s="310" t="str">
-        <x:v>执行中计划正常MQTT实测点经PostGIS返回WITHIN/OUTSIDE，页面分别绿色/红色，未飞计划线保持灰色。独立轨迹证据页没有匹配航线依据时显示黄色关系未知及明确说明；后端缺航线与缺间隔回归通过，不用未知数据染成符合。</x:v>
+        <x:v>正常API确认事件，模拟外部调用延迟期间短信SENDING且尝试1次；强制终止后端进程并重启，原60秒租约内保持SENDING，过期转UNKNOWN，仍1次且0送达记录，电话WAITING；页面明确须对账、禁止盲目补发。异常配置已撤销，健康接口200。</x:v>
       </x:c>
       <x:c r="F218" s="310" t="str">
-        <x:v>qa-r12/trajectory-final.json; trajectory-red-green-grey-ui.png; same-name-evidence-b-loaded.txt; same-name-evidence-b.png; rule-param-green.log</x:v>
+        <x:v>qa-r12/advisory-restart-sending.json; advisory-restart-sending-ui.txt; advisory-restart-recovered.json; advisory-restart-stable.json; advisory-restart-recovered-ui.txt; advisory-restart-recovered.png</x:v>
       </x:c>
       <x:c r="G218" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21123,16 +21129,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C219" s="310" t="str">
-        <x:v>主清单 126</x:v>
+        <x:v>主清单 81</x:v>
       </x:c>
       <x:c r="D219" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E219" s="310" t="str">
-        <x:v>既有空态、加载、401/403/404/500/超时和恢复证据基础上，实际复核表单验证改判未选结论、1001字说明均阻止提交并明确错误；真实POST响应延迟期间按钮禁用且显示正在处理，释放后仅1条复核/版本1，无重复提交或失败成功提示。</x:v>
+        <x:v>实际页面驳回曾500，追加迁移010修复后原表单成功；另一有权账号批准200，申请人自批409，旧版本重批409。实际审批人及时间保存、驳回无有效期。</x:v>
       </x:c>
       <x:c r="F219" s="310" t="str">
-        <x:v>qa-r12/ui-error-*.txt; ui-fault-test-summary.json; review-required-validation.txt; review-length-validation.txt; review-submit-disabled.txt; review-confirmed-ui.txt; review-state-transitions.json</x:v>
+        <x:v>qa-r12/approval-rejection-cancellation.json; rejection-fixed.png; rejection-green-package.log</x:v>
       </x:c>
       <x:c r="G219" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21146,16 +21152,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C220" s="310" t="str">
-        <x:v>主清单 106</x:v>
+        <x:v>主清单 83</x:v>
       </x:c>
       <x:c r="D220" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E220" s="310" t="str">
-        <x:v>无办理权限账号可读获准移送材料，但下载原件、冻结、发送通知均403；无查看权限分支沿用本轮真实受限角色API403及直链拒绝证据。修复证据冻结/解冻/销毁入口权限遗漏，6项回归、构建扫描及浏览器禁用提示验证通过。此项按无办理权限分支验收，不代表跨组织范围正样本已补齐。</x:v>
+        <x:v>此前已以有效观测验证自然到期AUTHORIZATION_EXPIRED、撤销/驳回INVALID_TRANSITION。补测通过CDP只替换一次详情来模拟旧按钮，执行接口与回读使用真实后端；三种终止状态均409，当前因观测过期先返回ADVISORY_COUNTER_BLOCKED，授权内容/版本前后完全一致。发现并修复错误弹窗仍声称已批准的问题：回读非APPROVED即关闭旧表单并提示真实状态。6项反例回归、build/scan、双端口重启200及三状态浏览器复测通过。</x:v>
       </x:c>
       <x:c r="F220" s="310" t="str">
-        <x:v>qa-r12/evidence-permission-api.json; handoff-readonly-ui.txt; evidence-readonly-before.txt; evidence-readonly-after.txt; evidence-readonly-fixed.png; restricted-apis.json; evidence-permission.test.cjs; evidence-permission-build.log</x:v>
+        <x:v>qa-r12/natural-expiry.json; cancelled-execute.json; stale-execution-current.json; stale-execution-after.json; stale-execution-*-fixed-response.json; stale-execution-*-fixed-ui.txt; stale-execution-green.log</x:v>
       </x:c>
       <x:c r="G220" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21169,16 +21175,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C221" s="310" t="str">
-        <x:v>主清单 74</x:v>
+        <x:v>主清单 84</x:v>
       </x:c>
       <x:c r="D221" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E221" s="310" t="str">
-        <x:v>补齐仅 local+qa / mock-replay / 精确事件生效的异常模拟入口；SENT 短信保持 UNKNOWN、0送达记录；NO_ANSWER 与 ANSWERED 未播完均 UNKNOWN、各1次，不写播放完成时间、不启动播放后观察、不显示反制入口。浏览器与正常API均核对。</x:v>
+        <x:v>临时显式DIRECT操作员经当前双源观测、关联违规研判发起，本机10007 CM4实际回码完成；自动干扰续链保留同一真实发起人，approved_by缺省。UI直接操作人正确、审批人不适用。仅协议模拟，非射频验收。</x:v>
       </x:c>
       <x:c r="F221" s="310" t="str">
-        <x:v>qa-r12/advisory-sent-result.json；advisory-noanswer-result.json；advisory-noanswer-ui.txt；advisory-answered-phase-fixed.json；advisory-answered-fixed-expanded-ui.txt</x:v>
+        <x:v>qa-r12/counter-r20/direct-start.json; direct-result.json; direct-ui.txt; cm4-independent.log</x:v>
       </x:c>
       <x:c r="G221" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21192,16 +21198,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C222" s="310" t="str">
-        <x:v>主清单 79</x:v>
+        <x:v>主清单 88</x:v>
       </x:c>
       <x:c r="D222" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E222" s="310" t="str">
-        <x:v>正常API确认事件，模拟外部调用延迟期间短信SENDING且尝试1次；强制终止后端进程并重启，原60秒租约内保持SENDING，过期转UNKNOWN，仍1次且0送达记录，电话WAITING；页面明确须对账、禁止盲目补发。异常配置已撤销，健康接口200。</x:v>
+        <x:v>经正常DIRECT API创建实际QUEUED四通道指令后，分别撤DIRECT/设备权限、停用用户/角色、撤范围、授权过期、观测超过当前配置窗口；H2/PG各7项均CANCELLED，重复dispatch无issued_at、无回执、仍仅一条命令。另覆盖普通审批排队过期。仅隔离软件队列验收，不代表现场设备验收。</x:v>
       </x:c>
       <x:c r="F222" s="310" t="str">
-        <x:v>qa-r12/advisory-restart-sending.json; advisory-restart-sending-ui.txt; advisory-restart-recovered.json; advisory-restart-stable.json; advisory-restart-recovered-ui.txt; advisory-restart-recovered.png</x:v>
+        <x:v>qa-r12/direct-queued-eligibility-final.log;fix51-queue-final.log</x:v>
       </x:c>
       <x:c r="G222" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21215,16 +21221,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C223" s="310" t="str">
-        <x:v>主清单 44</x:v>
+        <x:v>主清单 93</x:v>
       </x:c>
       <x:c r="D223" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E223" s="310" t="str">
-        <x:v>已通过正常分类修订API将独立QA无人机改判BIRD，原无人机深链清空详情且UAV列表不再包含该目标；另在浏览器精准阻断关联告警GET，页面明确网络失败，无核实入口，返回研判仍保留并入既有告警与前往告警入口，不按无告警放开重复复核。故障注入已解除。</x:v>
+        <x:v>设备通道授权0009批准后、执行前撤销；刷新/重开仍已撤销无执行入口。上一轮真实协议急停0005重开并刷新仍反制已中止、allowed_actions为空，未恢复命令或授权。</x:v>
       </x:c>
       <x:c r="F223" s="310" t="str">
-        <x:v>qa-r12/classification-change.json; classification-uav-before.txt; classification-non-uav-after.txt; associated-alarm-read-failed-ui.txt; associated-alarm-return-legality-ui.txt; associated-alarm-return-more-ui.txt</x:v>
+        <x:v>qa-r12/approval-rejection-cancellation.json; stopped-task-reopened.txt; stopped-task-refreshed.txt; cancelled-task-reopened.txt; stop-cancel-final-state.json</x:v>
       </x:c>
       <x:c r="G223" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21238,16 +21244,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C224" s="310" t="str">
-        <x:v>主清单 147</x:v>
+        <x:v>主清单 94</x:v>
       </x:c>
       <x:c r="D224" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E224" s="310" t="str">
-        <x:v>实际浏览器保存并启用QA规则，执行引擎保持DISABLED、运行记录0、待核实事件未自动推进；管理端页内及编辑提示已修复为不会触发动作。管理员仍可在业务前台人工核实（留下真实操作者历史），只读账号相同动作403。测试规则已停用，管理端138项测试、lint/build通过，重启5175且HTTP200。</x:v>
+        <x:v>本机CM4真实TCP接收后丢弃全关回码：急停保持FAILED且未声称停机；重复急停复用原stop/command，显式重试同键仅一条新指令，全关ACK仍待现场核查。PostgreSQL并发、迟到原命令和旧链隔离回归通过；修复反馈被隐藏并完成实际页面补原因、空核查依据禁用验证。仅本机协议模拟。 追加错回码0xf冒充全关的反例修复：65项回归及实际API均拒绝成功；成功回执0。</x:v>
       </x:c>
       <x:c r="F224" s="310" t="str">
-        <x:v>qa-r12/automation-disabled-saved.json; automation-disabled-editor.txt; automation-disabled-saved-ui.txt; automation-disabled-manual-before.json; automation-disabled-manual-after.json; automation-disabled-manual-success-ui.txt; automation-test-rule-disabled.json; admin-rule-tests.log</x:v>
+        <x:v>qa-r12/counter-r20/stop-race-fixed.json; stop-failure-repeated.json; stop-retry-final.json; stop-race-green-package.log; emergency-stop-feedback-fixed-ui.txt; emergency-stop-ui-after.json; emergency-stop-feedback.test.cjs; counter-r22/wrong-state.json; counter-r22/late-reply.json; counter-reply-final-package.log</x:v>
       </x:c>
       <x:c r="G224" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21261,16 +21267,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C225" s="310" t="str">
-        <x:v>主清单 102</x:v>
+        <x:v>主清单 95</x:v>
       </x:c>
       <x:c r="D225" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E225" s="310" t="str">
-        <x:v>修复模拟通知被前端一律只读的问题，遵循后端can_notify及原模拟环境门禁。正常API建立独立交接，页面完成未发送→SUBMITTED，未知重发409；受限模拟明确FAILED后页面补发，仅新增一次投递，再次UNKNOWN禁止重发。三次历史完整，模拟标识及确认提示保留，测试绑定已停用。4项反例回归、build/scan及5173/5177重启200通过。</x:v>
+        <x:v>正常MQTT观测、模拟防控空域及同事件充分研判补齐21条待审批。审批账号实际页面20+1跨页、返回无重复遗漏；一次只读503明确报错，恢复重读21条。直接调用readPending验证101条跨接口页及失败/变总数/重复/空缺页均正确拒绝不完整结果。21条全部撤销并在全部记录显示历史，后端待审批为0；临时角色已恢复、空域已撤回、发布器自然退出。无设备执行。</x:v>
       </x:c>
       <x:c r="F225" s="310" t="str">
-        <x:v>qa-r12/handoff-ui-sample-created.json; handoff-ui-ready.json; handoff-ui-initial-confirm.txt; handoff-ui-pending-no-repeat.json; handoff-ui-explicit-failure.json; handoff-ui-failed-retry-enabled.txt; handoff-ui-retry-complete.json; handoff-ui-retry-end.txt; handoff-notification-green.log</x:v>
+        <x:v>qa-r12/pending-pagination-created.json; pending-pagination-page1.txt; pending-pagination-page2.txt; pending-pagination-read-failure.txt; pending-pagination-recovered.txt; pending-pagination-boundaries.json; pending-pagination-all-cancelled.txt; pending-pagination-after.json; pending-pagination-cleanup.json</x:v>
       </x:c>
       <x:c r="G225" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21307,16 +21313,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C227" s="310" t="str">
-        <x:v>主清单 83</x:v>
+        <x:v>主清单 100</x:v>
       </x:c>
       <x:c r="D227" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E227" s="310" t="str">
-        <x:v>此前已以有效观测验证自然到期AUTHORIZATION_EXPIRED、撤销/驳回INVALID_TRANSITION。补测通过CDP只替换一次详情来模拟旧按钮，执行接口与回读使用真实后端；三种终止状态均409，当前因观测过期先返回ADVISORY_COUNTER_BLOCKED，授权内容/版本前后完全一致。发现并修复错误弹窗仍声称已批准的问题：回读非APPROVED即关闭旧表单并提示真实状态。6项反例回归、build/scan、双端口重启200及三状态浏览器复测通过。</x:v>
+        <x:v>同一真实模拟交接依次验证待发送、送达待确认、发送失败、已送达；原3次尝试分别保留PENDING_DELIVERY、FAILED、DELIVERED，页面查询不发送，未知不能算成功。</x:v>
       </x:c>
       <x:c r="F227" s="310" t="str">
-        <x:v>qa-r12/natural-expiry.json; cancelled-execute.json; stale-execution-current.json; stale-execution-after.json; stale-execution-*-fixed-response.json; stale-execution-*-fixed-ui.txt; stale-execution-green.log</x:v>
+        <x:v>qa-r12/handoff-pending-ui.txt; handoff-submitted-ui.txt; handoff-failed-ui.txt; handoff-delivered-timeout-ui.txt; handoff-receipt-invariants.json</x:v>
       </x:c>
       <x:c r="G227" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21330,16 +21336,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C228" s="310" t="str">
-        <x:v>主清单 135</x:v>
+        <x:v>主清单 101</x:v>
       </x:c>
       <x:c r="D228" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E228" s="310" t="str">
-        <x:v>经正常业务API为18条既有已核实回放告警创建交接，加既有3条共21项；通知配置过期故新增记录真实保持待发送。处罚收件箱第1页24条投递、第2页1条已送达历史，前后页无重复，末页不可再翻；已收到与其他发送分开。短信18/电话9/风险4条均浏览器打开刷新，网络只有GET；全部记录和第二页前后完全一致，无发送/拨号/签收副作用。</x:v>
+        <x:v>未进入签收、等待签收、回执超时及已签收分别验证；迟到送达后保留送达时间，签收超时不抹掉送达。最终已签收但页面仍显示暂无关联案件结果，不认定处罚完成。</x:v>
       </x:c>
       <x:c r="F228" s="310" t="str">
-        <x:v>qa-r12/inbox-pagination-created.json; inbox-pagination-before.json; inbox-pagination-page1.txt; inbox-pagination-page2.txt; inbox-pagination-readonly-requests.json; inbox-pagination-after.json</x:v>
+        <x:v>qa-r12/handoff-receipt-sequence.json; handoff-timeout-ui.txt; handoff-delivered-timeout-ui.txt; handoff-acknowledged-ui.txt</x:v>
       </x:c>
       <x:c r="G228" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21353,16 +21359,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C229" s="310" t="str">
-        <x:v>主清单 29</x:v>
+        <x:v>主清单 102</x:v>
       </x:c>
       <x:c r="D229" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E229" s="310" t="str">
-        <x:v>完全覆盖、部分覆盖、无覆盖已使用正常API计划和预报在浏览器验证。缺时间作为防御分支，以CDP只改一次详情响应start_at/end_at为null，实际天气接口保持真实；页面显示计划飞行时段不完整/无法确定对应预报时段，不展示任意时段。后台计划前后完全一致，拦截清除并重载真实页面。</x:v>
+        <x:v>修复模拟通知被前端一律只读的问题，遵循后端can_notify及原模拟环境门禁。正常API建立独立交接，页面完成未发送→SUBMITTED，未知重发409；受限模拟明确FAILED后页面补发，仅新增一次投递，再次UNKNOWN禁止重发。三次历史完整，模拟标识及确认提示保留，测试绑定已停用。4项反例回归、build/scan及5173/5177重启200通过。</x:v>
       </x:c>
       <x:c r="F229" s="310" t="str">
-        <x:v>qa-r12/weather-full.txt; weather-partial.txt; weather-none.txt; weather-coverage-plans.json; weather-missing-time-source.json; weather-missing-time-ui.txt; weather-missing-time.png</x:v>
+        <x:v>qa-r12/handoff-ui-sample-created.json; handoff-ui-ready.json; handoff-ui-initial-confirm.txt; handoff-ui-pending-no-repeat.json; handoff-ui-explicit-failure.json; handoff-ui-failed-retry-enabled.txt; handoff-ui-retry-complete.json; handoff-ui-retry-end.txt; handoff-notification-green.log</x:v>
       </x:c>
       <x:c r="G229" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21376,16 +21382,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C230" s="310" t="str">
-        <x:v>主清单 121</x:v>
+        <x:v>主清单 103</x:v>
       </x:c>
       <x:c r="D230" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E230" s="310" t="str">
-        <x:v>已覆盖真实空统计与全零趋势；浏览器通过只读模拟响应加入两条长分类，发现环图图例省略号截断并修复。StatsPage.drawCharts改为完整换行及零分母0.0%，全零不绘制虚构的等分扇区。3项回归、build/scan、重启双端口HTTP200通过；默认、实际CSS1280x720/1366x768/1440x900核验，文档无横向溢出。夹具与视口覆盖已清除，恢复真实数据。</x:v>
+        <x:v>旧投递的迟到回执409，当前投递迟到送达可接受；成功不能回退失败409。重复签收同版本4重放不增长，夹带另一交接ID不改变真实关联，另一记录不变。</x:v>
       </x:c>
       <x:c r="F230" s="310" t="str">
-        <x:v>qa-r12/stats-long-name-before.png; stats-long-name-fixed.png; stats-long-name-1280.png; stats-zero-fixed.png; stats-label-viewports.json; stats-long-label-green.log</x:v>
+        <x:v>qa-r12/handoff-receipt-sequence.json; handoff-receipt-invariants.json</x:v>
       </x:c>
       <x:c r="G230" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21399,16 +21405,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C231" s="310" t="str">
-        <x:v>主清单 95</x:v>
+        <x:v>主清单 106</x:v>
       </x:c>
       <x:c r="D231" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E231" s="310" t="str">
-        <x:v>正常MQTT观测、模拟防控空域及同事件充分研判补齐21条待审批。审批账号实际页面20+1跨页、返回无重复遗漏；一次只读503明确报错，恢复重读21条。直接调用readPending验证101条跨接口页及失败/变总数/重复/空缺页均正确拒绝不完整结果。21条全部撤销并在全部记录显示历史，后端待审批为0；临时角色已恢复、空域已撤回、发布器自然退出。无设备执行。</x:v>
+        <x:v>无办理权限账号可读获准移送材料，但下载原件、冻结、发送通知均403；无查看权限分支沿用本轮真实受限角色API403及直链拒绝证据。修复证据冻结/解冻/销毁入口权限遗漏，6项回归、构建扫描及浏览器禁用提示验证通过。此项按无办理权限分支验收，不代表跨组织范围正样本已补齐。</x:v>
       </x:c>
       <x:c r="F231" s="310" t="str">
-        <x:v>qa-r12/pending-pagination-created.json; pending-pagination-page1.txt; pending-pagination-page2.txt; pending-pagination-read-failure.txt; pending-pagination-recovered.txt; pending-pagination-boundaries.json; pending-pagination-all-cancelled.txt; pending-pagination-after.json; pending-pagination-cleanup.json</x:v>
+        <x:v>qa-r12/evidence-permission-api.json; handoff-readonly-ui.txt; evidence-readonly-before.txt; evidence-readonly-after.txt; evidence-readonly-fixed.png; restricted-apis.json; evidence-permission.test.cjs; evidence-permission-build.log</x:v>
       </x:c>
       <x:c r="G231" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21422,16 +21428,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C232" s="310" t="str">
-        <x:v>主清单 40</x:v>
+        <x:v>主清单 113</x:v>
       </x:c>
       <x:c r="D232" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E232" s="310" t="str">
-        <x:v>既有CONFIRMED/REJECTED/OVERRIDDEN服务端和页面筛选已核对。本轮正常回放观测形成21条SUFFICIENT、review_required=false、review PENDING_REVIEW/version0记录；固定15秒窗口未复核记录3条，needs_review=true为0，false为3。页面非法21条切待复核为0，未把所有从未人工操作的记录归入待复核。DEMO参数警示保留；仅验筛选逻辑，不代表参数或算法准确性验收。</x:v>
+        <x:v>在真实任务视频读取时分别暂停告警、研判、反制GET，然后离页；三个请求均随卸载取消，释放拦截后video=0，无旧画面回挂；态势换目标也清理旧流。拦截已解除。</x:v>
       </x:c>
       <x:c r="F232" s="310" t="str">
-        <x:v>qa-r12/review-state-transitions.json; review-filter-api.json; review-needs-latest.json; review-filter-confirmed.txt; review-filter-rejected.txt; review-filter-overridden.txt; review-not-required-positive.json; review-not-required-detail.json; review-not-required-before.txt; review-not-required-filtered.txt</x:v>
+        <x:v>qa-r12/video-r18/alarm-delayed-leave.txt; legality-delayed-leave.txt; authorization-delayed-leave.txt; situation-switched.txt</x:v>
       </x:c>
       <x:c r="G232" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21445,16 +21451,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C233" s="310" t="str">
-        <x:v>主清单 21</x:v>
+        <x:v>主清单 121</x:v>
       </x:c>
       <x:c r="D233" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E233" s="310" t="str">
-        <x:v>态势页真实本地HLS播放后收起video=0，切目标038清除旧039画面，离页释放；无任务明确说明，真实只读账号UI无权限且API403，测试画面标识保留。</x:v>
+        <x:v>已覆盖真实空统计与全零趋势；浏览器通过只读模拟响应加入两条长分类，发现环图图例省略号截断并修复。StatsPage.drawCharts改为完整换行及零分母0.0%，全零不绘制虚构的等分扇区。3项回归、build/scan、重启双端口HTTP200通过；默认、实际CSS1280x720/1366x768/1440x900核验，文档无横向溢出。夹具与视口覆盖已清除，恢复真实数据。</x:v>
       </x:c>
       <x:c r="F233" s="310" t="str">
-        <x:v>qa-r12/video-r18/situation-playing.png; situation-switched.txt; reader-situation-no-permission.txt; reader-video-permission.json</x:v>
+        <x:v>qa-r12/stats-long-name-before.png; stats-long-name-fixed.png; stats-long-name-1280.png; stats-zero-fixed.png; stats-label-viewports.json; stats-long-label-green.log</x:v>
       </x:c>
       <x:c r="G233" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21468,16 +21474,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C234" s="310" t="str">
-        <x:v>主清单 48</x:v>
+        <x:v>主清单 124</x:v>
       </x:c>
       <x:c r="D234" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E234" s="310" t="str">
-        <x:v>正常API发起039目标光电跟踪，实际MQTT BeginTracking回包，设备/目标/任务吻合；命令成功、TRACKING与HLS可用分别验证，960x540视频实际播放；结束MQTT回执后ENDED及旧HLS404。仅本地模拟验收。</x:v>
+        <x:v>真实 MQTT workState=2→1，设备异常→在线，页面同一选中设备自动更新；整体健康仍UNKNOWN。当前测试页以浏览器媒体仿真启用prefers-reduced-motion，实际绘图函数常量静态红光22.5；普通模式6/17/28变化，恢复后不再应用红光。未改操作系统设置，测试后媒体仿真已撤销。</x:v>
       </x:c>
       <x:c r="F234" s="310" t="str">
-        <x:v>qa-r12/video-r18/business-started.json; business-player-proof.json; business-fixed-video.json; business-final.json; cleanup.json</x:v>
+        <x:v>qa-r12/motion-fault-api.json; motion-restored-api.json; motion-fault-ui.png; motion-restored-ui.png; motion-media-state.json; motion-function-verification.json</x:v>
       </x:c>
       <x:c r="G234" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21491,16 +21497,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C235" s="310" t="str">
-        <x:v>主清单 65</x:v>
+        <x:v>主清单 126</x:v>
       </x:c>
       <x:c r="D235" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E235" s="310" t="str">
-        <x:v>告警与反制详情默认展开实际测试HLS，收起video=0再展开；无任务、真实无权限、单次503分别提示；查看前后授权REQUESTED/version0一致，不触发反制。</x:v>
+        <x:v>既有空态、加载、401/403/404/500/超时和恢复证据基础上，实际复核表单验证改判未选结论、1001字说明均阻止提交并明确错误；真实POST响应延迟期间按钮禁用且显示正在处理，释放后仅1条复核/版本1，无重复提交或失败成功提示。</x:v>
       </x:c>
       <x:c r="F235" s="310" t="str">
-        <x:v>qa-r12/video-r18/alarm-default-expanded.txt; authorization-video-expanded.txt; authorization-video-failed.txt; reader-authorization-no-permission.txt; authorization-before-view.json; authorization-after-view.json</x:v>
+        <x:v>qa-r12/ui-error-*.txt; ui-fault-test-summary.json; review-required-validation.txt; review-length-validation.txt; review-submit-disabled.txt; review-confirmed-ui.txt; review-state-transitions.json</x:v>
       </x:c>
       <x:c r="G235" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21514,16 +21520,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C236" s="310" t="str">
-        <x:v>主清单 113</x:v>
+        <x:v>主清单 134</x:v>
       </x:c>
       <x:c r="D236" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E236" s="310" t="str">
-        <x:v>在真实任务视频读取时分别暂停告警、研判、反制GET，然后离页；三个请求均随卸载取消，释放拦截后video=0，无旧画面回挂；态势换目标也清理旧流。拦截已解除。</x:v>
+        <x:v>四策略已分别验证：短信撤离LEFT且无电话、电话后10秒LEFT、持续飞行待反制、短信停报UNKNOWN且不拨号；全部MOCK/replay，无真实通知。</x:v>
       </x:c>
       <x:c r="F236" s="310" t="str">
-        <x:v>qa-r12/video-r18/alarm-delayed-leave.txt; legality-delayed-leave.txt; authorization-delayed-leave.txt; situation-switched.txt</x:v>
+        <x:v>qa-r12/sms-departure-fixed.json; voice-departure-fixed.json; drop-sms-fixed.json</x:v>
       </x:c>
       <x:c r="G236" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21537,16 +21543,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C237" s="310" t="str">
-        <x:v>主清单 56</x:v>
+        <x:v>主清单 135</x:v>
       </x:c>
       <x:c r="D237" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E237" s="310" t="str">
-        <x:v>通过受限本地QA入口新增纯气象风险，实际时钟自然到期后CURRENT→UNKNOWN，核验/通知历史及版本不变；已过期天气和缺少新观测的鸟群风险均显示待确认，不视为解除。未来预警到时前不计当前。</x:v>
+        <x:v>经正常业务API为18条既有已核实回放告警创建交接，加既有3条共21项；通知配置过期故新增记录真实保持待发送。处罚收件箱第1页24条投递、第2页1条已送达历史，前后页无重复，末页不可再翻；已收到与其他发送分开。短信18/电话9/风险4条均浏览器打开刷新，网络只有GET；全部记录和第二页前后完全一致，无发送/拨号/签收副作用。</x:v>
       </x:c>
       <x:c r="F237" s="310" t="str">
-        <x:v>qa-r12/weather-risk-natural-expiry.json; weather-risk-three-boundaries.json; weather-vs-nonweather-current.json; weather-current-plan-expired.txt; weather-risk-package-final.log</x:v>
+        <x:v>qa-r12/inbox-pagination-created.json; inbox-pagination-before.json; inbox-pagination-page1.txt; inbox-pagination-page2.txt; inbox-pagination-readonly-requests.json; inbox-pagination-after.json</x:v>
       </x:c>
       <x:c r="G237" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21560,16 +21566,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C238" s="310" t="str">
-        <x:v>主清单 84</x:v>
+        <x:v>主清单 137</x:v>
       </x:c>
       <x:c r="D238" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E238" s="310" t="str">
-        <x:v>临时显式DIRECT操作员经当前双源观测、关联违规研判发起，本机10007 CM4实际回码完成；自动干扰续链保留同一真实发起人，approved_by缺省。UI直接操作人正确、审批人不适用。仅协议模拟，非射频验收。</x:v>
+        <x:v>页面暂停8秒发送计数和模拟进度不变，继续后增长；停止批次STOPPED。真实进程重启复现并修复中文批次丢失及进度未落盘；重启保留47秒136条且不续发。纯MQTT撤权后继续发送缺陷修复后约2秒自动停在58条；重新登录不自动恢复。</x:v>
       </x:c>
       <x:c r="F238" s="310" t="str">
-        <x:v>qa-r12/counter-r20/direct-start.json; direct-result.json; direct-ui.txt; cm4-independent.log</x:v>
+        <x:v>qa-r12/simulator-control-samples.json; simulator-restart-fixed.png; simulator-session-expired-fixed.png; runtime-recovery-green-utf8.log; runtime-recovery-green-ansi.log; simulator-all-tests-final.log</x:v>
       </x:c>
       <x:c r="G238" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21583,16 +21589,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C239" s="310" t="str">
-        <x:v>主清单 94</x:v>
+        <x:v>主清单 138</x:v>
       </x:c>
       <x:c r="D239" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E239" s="310" t="str">
-        <x:v>本机CM4真实TCP接收后丢弃全关回码：急停保持FAILED且未声称停机；重复急停复用原stop/command，显式重试同键仅一条新指令，全关ACK仍待现场核查。PostgreSQL并发、迟到原命令和旧链隔离回归通过；修复反馈被隐藏并完成实际页面补原因、空核查依据禁用验证。仅本机协议模拟。 追加错回码0xf冒充全关的反例修复：65项回归及实际API均拒绝成功；成功回执0。</x:v>
+        <x:v>失效会话401回登录、无权限403明确拒绝、不存在计划404显示不存在、单请求500显示内部错误、实际15秒超时408分别核实；清除测试拦截后正常读取37条研判，不把异常当暂无数据。</x:v>
       </x:c>
       <x:c r="F239" s="310" t="str">
-        <x:v>qa-r12/counter-r20/stop-race-fixed.json; stop-failure-repeated.json; stop-retry-final.json; stop-race-green-package.log; emergency-stop-feedback-fixed-ui.txt; emergency-stop-ui-after.json; emergency-stop-feedback.test.cjs; counter-r22/wrong-state.json; counter-r22/late-reply.json; counter-reply-final-package.log</x:v>
+        <x:v>qa-r12/permission-revocation.json; legality-no-alarm-permission-api.json; ui-error-404.txt; ui-error-500.txt; ui-error-timeout.txt; ui-error-recovered.txt; ui-fault-test-summary.json</x:v>
       </x:c>
       <x:c r="G239" s="310" t="str">
         <x:v>完整条目通过</x:v>
@@ -21606,18 +21612,340 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="C240" s="310" t="str">
-        <x:v>主清单 26</x:v>
+        <x:v>主清单 141</x:v>
       </x:c>
       <x:c r="D240" s="310" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E240" s="310" t="str">
-        <x:v>独立PostgreSQL/PostGIS同一到时执行计划未匹配目标：正常GOOD显示疑似未按计划起飞；BAD显示设备异常、是否起飞待确认；UNKNOWN显示信息不完整。真实前台三分支与API结论一致，不以无目标认定未起飞。</x:v>
+        <x:v>两个独立人员会话并发核实、审批与撤销，均一方成功、另一方409版本冲突；旧审批页提交后自动回读已撤销，无覆盖。</x:v>
       </x:c>
       <x:c r="F240" s="310" t="str">
-        <x:v>qa-r12/maintenance-browser/postgres-fifth/normal-api.json；maintenance-browser/postgres-fifth/normal-ui.txt；maintenance-browser/postgres-fifth/unknown-api.json；maintenance-browser/postgres-fifth/unknown-ui.txt；maintenance-browser/postgres-fifth/abnormal-api.json；maintenance-browser/postgres-fifth/abnormal-ui.txt；due-plan-matrix-fixed-preflight.log</x:v>
+        <x:v>qa-r12/concurrent-verification.json; approval-cancel-race.json; stale-approval-cancelled.txt</x:v>
       </x:c>
       <x:c r="G240" s="310" t="str">
+        <x:v>完整条目通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="241" ht="100" customHeight="1">
+      <x:c r="A241" s="310" t="str">
+        <x:v>第十二轮</x:v>
+      </x:c>
+      <x:c r="B241" s="310" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="C241" s="310" t="str">
+        <x:v>主清单 147</x:v>
+      </x:c>
+      <x:c r="D241" s="310" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="E241" s="310" t="str">
+        <x:v>实际浏览器保存并启用QA规则，执行引擎保持DISABLED、运行记录0、待核实事件未自动推进；管理端页内及编辑提示已修复为不会触发动作。管理员仍可在业务前台人工核实（留下真实操作者历史），只读账号相同动作403。测试规则已停用，管理端138项测试、lint/build通过，重启5175且HTTP200。</x:v>
+      </x:c>
+      <x:c r="F241" s="310" t="str">
+        <x:v>qa-r12/automation-disabled-saved.json; automation-disabled-editor.txt; automation-disabled-saved-ui.txt; automation-disabled-manual-before.json; automation-disabled-manual-after.json; automation-disabled-manual-success-ui.txt; automation-test-rule-disabled.json; admin-rule-tests.log</x:v>
+      </x:c>
+      <x:c r="G241" s="310" t="str">
+        <x:v>完整条目通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="242" ht="100" customHeight="1">
+      <x:c r="A242" s="310" t="str">
+        <x:v>第十二轮</x:v>
+      </x:c>
+      <x:c r="B242" s="310" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="C242" s="310" t="str">
+        <x:v>主清单 90</x:v>
+      </x:c>
+      <x:c r="D242" s="310" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="E242" s="310" t="str">
+        <x:v>本机模拟完整覆盖占用、离线、故障：页面分别说明具体受阻，不走人工填写成功；H2/PG三种活动指令状态阻止第二事件启动，两账号两事件真实PG并发仅1启动。停用/离线无指令，排队变更取消且无发送时刻/回执；同事件重复与并发沿用已核验证据。停止/全关仍可排队。</x:v>
+      </x:c>
+      <x:c r="F242" s="310" t="str">
+        <x:v>qa-r12/counter-r20/stop-race-green-package.log; counter-r20/concurrent-direct.json; counter-boundaries-tests.log; fix52-53-final.log; fix52-fault-ui.png; fix52-fault-viewports.json; fix54-green.log; fix54-busy-ui.png; main90-offline-final.log; main90-offline-ui.png</x:v>
+      </x:c>
+      <x:c r="G242" s="310" t="str">
+        <x:v>完整条目通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="243" ht="100" customHeight="1">
+      <x:c r="A243" s="310" t="str">
+        <x:v>第十二轮</x:v>
+      </x:c>
+      <x:c r="B243" s="310" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="C243" s="310" t="str">
+        <x:v>主清单 87</x:v>
+      </x:c>
+      <x:c r="D243" s="310" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="E243" s="310" t="str">
+        <x:v>过期位置、合法、未知、证据不足、其他事件研判×申请/直接/执行三入口，H2与PostgreSQL共30项通过；追加新研判保留历史。隔离运行服务五种执行页面均明确本次没有下发，结束后5条授权仍APPROVED、EXECUTE事件0、设备指令0；未使用人工现场记录补资格。</x:v>
+      </x:c>
+      <x:c r="F243" s="310" t="str">
+        <x:v>qa-r12/main87-entry-matrix-final.log;main87-browser-frozen-clock.log;main87-manifest.json;main87-STALE.png;main87-LEGAL.png;main87-UNKNOWN.png;main87-INSUFFICIENT.png;main87-OTHER_EVENT.png</x:v>
+      </x:c>
+      <x:c r="G243" s="310" t="str">
+        <x:v>完整条目通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="244" ht="100" customHeight="1">
+      <x:c r="A244" s="310" t="str">
+        <x:v>第十二轮</x:v>
+      </x:c>
+      <x:c r="B244" s="310" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="C244" s="310" t="str">
+        <x:v>主清单 105</x:v>
+      </x:c>
+      <x:c r="D244" s="310" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="E244" s="310" t="str">
+        <x:v>H2/PG正式接口直接发起→停止授权→上传关联真实测试日志→移送→后补日志；旧快照全文不变，DIRECT保留原发起人且无审批人，后补证据仅追加事件关联。页面补显示冻结发起人与移送时证据，和当前关联证据分开；改名不改旧材料，精确链接打开before.txt，普通审批记录保留审批人。</x:v>
+      </x:c>
+      <x:c r="F244" s="310" t="str">
+        <x:v>qa-r12/main105-direct-frozen.log;main87-97-105-regression.log;fix55-before-ui.txt;fix55-after-ui.txt;fix55-final.png;fix55-viewports.json;fix55-frozen-link-ui.txt;fix55-ordinary-ui.txt;fix55-build-final.log;fix55-scan.log</x:v>
+      </x:c>
+      <x:c r="G244" s="310" t="str">
+        <x:v>完整条目通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="245" ht="100" customHeight="1">
+      <x:c r="A245" s="310" t="str">
+        <x:v>第十二轮</x:v>
+      </x:c>
+      <x:c r="B245" s="310" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="C245" s="310" t="str">
+        <x:v>主清单 97</x:v>
+      </x:c>
+      <x:c r="D245" s="310" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="E245" s="310" t="str">
+        <x:v>PG两起点三方并发及同键重放通过；独立运行服务三账号实际HTTP竞态分别形成EXECUTING/1命令和CANCELLED/0命令。第三请求确认等待PG事件锁时强制终止进程，数据库事务无新增；原库新进程重启后6个旧请求409，中断请求同键200且仅1命令，再重放409。办理历史与实际成功操作一致。</x:v>
+      </x:c>
+      <x:c r="F245" s="310" t="str">
+        <x:v>qa-r12/main87-97-105-regression.log;main97-http-races.json;main97-interrupted-http.json;main97-before-crash.json;main97-after-crash.json;main97-restart-replays.json;main97-after-replays.json;main97-summary.json;main97-process-restored.log</x:v>
+      </x:c>
+      <x:c r="G245" s="310" t="str">
+        <x:v>完整条目通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="246" ht="100" customHeight="1">
+      <x:c r="A246" s="310" t="str">
+        <x:v>第十二轮</x:v>
+      </x:c>
+      <x:c r="B246" s="310" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="C246" s="310" t="str">
+        <x:v>主清单 89</x:v>
+      </x:c>
+      <x:c r="D246" s="310" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="E246" s="310" t="str">
+        <x:v>实际回环MQTT与正式授权流程在H2/PG覆盖正常、撤直接权限、撤设备权限、撤范围和原授权到期。正常收到60003与60002两命令，子授权DIRECT、真实原发起人、无审批人、截止沿用原窗口；四阻断分支原命令COMPLETED但无子授权、实收仅1条。到期分支补新有效观测与研判，单独断言依据仍有效，排除观测过期误阻断。重复结算不重发。</x:v>
+      </x:c>
+      <x:c r="F246" s="310" t="str">
+        <x:v>qa-r12/counter-r20/stop-race-green-package.log; counter-r20/concurrent-direct.json; counter-boundaries-tests.log;fix51-red.log;fix51-green.log;fix51-queue-final.log;main89-91-wire-final.log;main89-91-wire/h2/;main89-91-wire/postgresql/</x:v>
+      </x:c>
+      <x:c r="G246" s="310" t="str">
+        <x:v>完整条目通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="247" ht="100" customHeight="1">
+      <x:c r="A247" s="310" t="str">
+        <x:v>第十二轮</x:v>
+      </x:c>
+      <x:c r="B247" s="310" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="C247" s="310" t="str">
+        <x:v>主清单 91</x:v>
+      </x:c>
+      <x:c r="D247" s="310" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="E247" s="310" t="str">
+        <x:v>无命令号CM4迟到不串任务/不重发已验。带msgNo凌云在H2/PG真实MQTT迟到成功失败归原任务，并发去重，不覆盖超时/取消或新命令；普通审批实际页面下发后仅1条60003，3秒超时，50秒后迟到成功保留FAILED与原历史且不续链。页面明确超时不代表未执行，从原授权精确查看原命令，返回仍失败、无执行入口。</x:v>
+      </x:c>
+      <x:c r="F247" s="310" t="str">
+        <x:v>qa-r12/counter-r22/late-reply.json; counter-r22/cm4.log; counter-reply-final-package.log;fix56-red.log;fix56-regression-package.log;fix56-regression-package-final.log;fix56-browser-checks.json;fix56-final.png;fix56-viewports.json;main89-91-wire-final.log;main91-before-late.json;fix57-timeout-ui.txt;main91-late-linked-ui.txt;main91-late-linked.png;main91-late-authorization-unchanged.txt;fix57-viewports.json;main91-browser-fixture.log</x:v>
+      </x:c>
+      <x:c r="G247" s="310" t="str">
+        <x:v>完整条目通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="248" ht="100" customHeight="1">
+      <x:c r="A248" s="310" t="str">
+        <x:v>第十二轮</x:v>
+      </x:c>
+      <x:c r="B248" s="310" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="C248" s="310" t="str">
+        <x:v>主清单 61</x:v>
+      </x:c>
+      <x:c r="D248" s="310" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="E248" s="310" t="str">
+        <x:v>告警详情恢复只读折叠历史，冻结材料保留原观察、紧急标记和办理人，明确不作为当前依据；切换事件不残留，三个视口无溢出。H2/PG历史及停用接口44项通过，实际页面夹具1项通过。</x:v>
+      </x:c>
+      <x:c r="F248" s="310" t="str">
+        <x:v>qa-r12/main61-history-regression.log; main61-browser-fixture-final.log; main61-alarm-ui.txt; main61-frozen-ui.txt; main61-switched-ui.txt; fix59-viewports.json; main61-alarm.png</x:v>
+      </x:c>
+      <x:c r="G248" s="310" t="str">
+        <x:v>完整条目通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="249" ht="100" customHeight="1">
+      <x:c r="A249" s="310" t="str">
+        <x:v>第十二轮</x:v>
+      </x:c>
+      <x:c r="B249" s="310" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="C249" s="310" t="str">
+        <x:v>主清单 34</x:v>
+      </x:c>
+      <x:c r="D249" s="310" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="E249" s="310" t="str">
+        <x:v>隔离H2页面实际鸟群、气球、风筝、未知四类深链均提示无可见无人机研判且详情为空；全部列表只含2架UAV，无计划无人机保留。H2/PG过滤与同范围计数通过。气球/风筝依现有UNKNOWN+subtype契约，不新增类型。</x:v>
+      </x:c>
+      <x:c r="F249" s="310" t="str">
+        <x:v>qa-r12/main34-36-api-final.log; main34-deep-links.json; main34-{BIRD,BALLOON,KITE,UNKNOWN}-ui.txt; main34-uav-list-ui.txt</x:v>
+      </x:c>
+      <x:c r="G249" s="310" t="str">
+        <x:v>完整条目通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="250" ht="100" customHeight="1">
+      <x:c r="A250" s="310" t="str">
+        <x:v>第十二轮</x:v>
+      </x:c>
+      <x:c r="B250" s="310" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="C250" s="310" t="str">
+        <x:v>主清单 36</x:v>
+      </x:c>
+      <x:c r="D250" s="310" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="E250" s="310" t="str">
+        <x:v>H2/PG合法空分、非法0/99/空分四组明确充分结论均无需复核；浏览器可靠合法/非法显示系统自动判定、待处理0，人工纠正仅为更多操作的可选项。此为受控读取/展示契约验证，不是算法准确率验收。</x:v>
+      </x:c>
+      <x:c r="F250" s="310" t="str">
+        <x:v>qa-r12/main34-36-api-final.log; main36-{legal,illegal,attention,optional-correction}-ui.txt; main36-illegal.png; main34-36-browser.log</x:v>
+      </x:c>
+      <x:c r="G250" s="310" t="str">
+        <x:v>完整条目通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="251" ht="100" customHeight="1">
+      <x:c r="A251" s="310" t="str">
+        <x:v>第十二轮</x:v>
+      </x:c>
+      <x:c r="B251" s="310" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="C251" s="310" t="str">
+        <x:v>主清单 46</x:v>
+      </x:c>
+      <x:c r="D251" s="310" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="E251" s="310" t="str">
+        <x:v>隔离 PostgreSQL/PostGIS 中构造范围内、边界上、范围外目标；受限账号只见授权单位/区域的3个目标，选择空域后仅内点与边界2个，清空恢复3个。交叉单位/区域的同坐标目标列表不出现、详情404；前端平面算法与ST_Covers/ST_Touches一致。仅验证平面筛选与范围授权，不把位置关系当作违规结论。</x:v>
+      </x:c>
+      <x:c r="F251" s="310" t="str">
+        <x:v>qa-r12/main46-browser-corrected.log; main46-geometry-agreement.json; main46-all-ui.txt; main46-selected-ui.txt; main46-cleared-ui.txt; main46-selected.png</x:v>
+      </x:c>
+      <x:c r="G251" s="310" t="str">
+        <x:v>完整条目通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="252" ht="100" customHeight="1">
+      <x:c r="A252" s="310" t="str">
+        <x:v>第十二轮</x:v>
+      </x:c>
+      <x:c r="B252" s="310" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="C252" s="310" t="str">
+        <x:v>主清单 49</x:v>
+      </x:c>
+      <x:c r="D252" s="310" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="E252" s="310" t="str">
+        <x:v>隔离页面已验证无位置提示不能引导光电、无权限提示无法读取、忙设备提示没有可用空闲设备；三种情况均无开始跟踪入口。仅气象无目标风险不显示光电跟踪、不造目标。28项API回归+1浏览器夹具通过，结束时跟踪任务和设备指令数量均未增加。</x:v>
+      </x:c>
+      <x:c r="F252" s="310" t="str">
+        <x:v>qa-r12/main49-api-guards-final.log; main49-browser.log; main49-no-permission-ui.txt; main49-missing-ui.txt; main49-busy-ui.txt; main49-weather-ui.txt; main49-busy.png</x:v>
+      </x:c>
+      <x:c r="G252" s="310" t="str">
+        <x:v>完整条目通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="253" ht="100" customHeight="1">
+      <x:c r="A253" s="310" t="str">
+        <x:v>第十二轮</x:v>
+      </x:c>
+      <x:c r="B253" s="310" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="C253" s="310" t="str">
+        <x:v>主清单 145</x:v>
+      </x:c>
+      <x:c r="D253" s="310" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="E253" s="310" t="str">
+        <x:v>隔离PostGIS构造两个单位同名空域，甲单位含mock/replay/live三种来源。甲账号只见本单位3条且逐条打开编号正确；退出换乙账号只见乙单位1条，旧列表/详情不残留。模拟/回放独立标记，源模式API一致；双方访问另一单位详情均404。</x:v>
+      </x:c>
+      <x:c r="F253" s="310" t="str">
+        <x:v>qa-r12/main145-browser-final.log; main145-manifest.json; main145-account-a-ui.txt; main145-a-details.json; main145-account-b-ui.txt; main145-b-detail.txt; main145-account-a.png; main145-account-b.png</x:v>
+      </x:c>
+      <x:c r="G253" s="310" t="str">
+        <x:v>完整条目通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="254" ht="100" customHeight="1">
+      <x:c r="A254" s="310" t="str">
+        <x:v>第十二轮</x:v>
+      </x:c>
+      <x:c r="B254" s="310" t="str">
+        <x:v>2026-09-28</x:v>
+      </x:c>
+      <x:c r="C254" s="310" t="str">
+        <x:v>主清单 119</x:v>
+      </x:c>
+      <x:c r="D254" s="310" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="E254" s="310" t="str">
+        <x:v>隔离H2/PostgreSQL对开始前1ms、开始零点、结束日末1ms、次日零点六组目标/立案时间逐项验证。26回归通过；独立PostGIS浏览器实际两单日2/0、2/1及跨年两日4/1均正确，重复末次观测未新增计数；CSV接口200且总数4。仅使用一次性合成统计事实，不证明真实处罚结果；浏览器下载连接中断未另算下载通过。</x:v>
+      </x:c>
+      <x:c r="F254" s="310" t="str">
+        <x:v>qa-r12/main119-api.log; main119-browser-final.log; main119-manifest.json; main119-api-facts.json; main119-day1-ui.txt; main119-day2-ui.txt; main119-range-ui.txt; main119-api-export.csv</x:v>
+      </x:c>
+      <x:c r="G254" s="310" t="str">
         <x:v>完整条目通过</x:v>
       </x:c>
     </x:row>
@@ -21652,10 +21980,10 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="4">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73350748be7242fd"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd23be0aead964645"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82d0c54718874263"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R979ebe5b9504412a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf0d2521d4af4929"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6d307195d414818"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3c46373a7e6437c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac883e200e394345"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21863,7 +22191,7 @@
         <x:v>暂时测不了</x:v>
       </x:c>
       <x:c r="G8" s="303" t="str">
-        <x:v>第十一轮：已用独立QA账号通过正常API完成首次改密，验证旧密码及旧会话失效；页面改密全路径未重跑。</x:v>
+        <x:v>第十二轮：已补实际首次改密账号登录及直接打开统计页面，两次均跳转首次改密页；旧轮API已验证改密后旧密码/旧会话失效。浏览器工具要求用户亲自录入并提交新密码，因此未代做这一页面步骤，保留未完整状态。</x:v>
       </x:c>
       <x:c r="H8" s="303" t="str">
         <x:v>Codex</x:v>
@@ -21872,7 +22200,7 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J8" s="303" t="str">
-        <x:v>qa-r11/auth-first-change.json</x:v>
+        <x:v>qa-r12/main3-gate-ui.txt; main3-gate.png; main119-browser-final.log</x:v>
       </x:c>
       <x:c r="K8" s="303" t="str">
         <x:v>前置条件未齐</x:v>
@@ -22915,10 +23243,10 @@
         <x:v>182</x:v>
       </x:c>
       <x:c r="F39" s="303" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="G39" s="303" t="str">
-        <x:v>第十轮：实际鸟类目标022不进入无人机研判；鸟类/缺失目标直链均无残留UAV信息。当前协议编译器未提供气球/风筝枚举，未知类全分支未具备。</x:v>
+        <x:v>第十二轮：隔离H2页面实际鸟群、气球、风筝、未知四类深链均提示无可见无人机研判且详情为空；全部列表只含2架UAV，无计划无人机保留。H2/PG过滤与同范围计数通过。气球/风筝依现有UNKNOWN+subtype契约，不新增类型。</x:v>
       </x:c>
       <x:c r="H39" s="303" t="str">
         <x:v>Codex</x:v>
@@ -22927,11 +23255,9 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J39" s="303" t="str">
-        <x:v>bird-deeplink-fixed.txt；missing-target-deeplink.txt；scene-b-verify.json</x:v>
-      </x:c>
-      <x:c r="K39" s="303" t="str">
-        <x:v>BUG-016已修复；协议样本缺口</x:v>
-      </x:c>
+        <x:v>qa-r12/main34-36-api-final.log; main34-deep-links.json; main34-{BIRD,BALLOON,KITE,UNKNOWN}-ui.txt; main34-uav-list-ui.txt</x:v>
+      </x:c>
+      <x:c r="K39" s="303" t="str"/>
     </x:row>
     <x:row r="40" ht="160" customHeight="1">
       <x:c r="A40" s="153">
@@ -22983,10 +23309,10 @@
         <x:v>186</x:v>
       </x:c>
       <x:c r="F41" s="303" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="G41" s="303" t="str">
-        <x:v>第十轮：当前回放仍使用DEMO演示参数，缺依据充分且可明确判为合法的同批正向样本。</x:v>
+        <x:v>第十二轮：H2/PG合法空分、非法0/99/空分四组明确充分结论均无需复核；浏览器可靠合法/非法显示系统自动判定、待处理0，人工纠正仅为更多操作的可选项。此为受控读取/展示契约验证，不是算法准确率验收。</x:v>
       </x:c>
       <x:c r="H41" s="303" t="str">
         <x:v>Codex</x:v>
@@ -22995,11 +23321,9 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J41" s="303" t="str">
-        <x:v>第十轮报告；本轮回放/页面/隔离回归证据</x:v>
-      </x:c>
-      <x:c r="K41" s="303" t="str">
-        <x:v>场景或环境前置条件未齐</x:v>
-      </x:c>
+        <x:v>qa-r12/main34-36-api-final.log; main36-{legal,illegal,attention,optional-correction}-ui.txt; main36-illegal.png; main34-36-browser.log</x:v>
+      </x:c>
+      <x:c r="K41" s="303" t="str"/>
     </x:row>
     <x:row r="42" ht="160" customHeight="1">
       <x:c r="A42" s="153">
@@ -23329,10 +23653,10 @@
         <x:v>217</x:v>
       </x:c>
       <x:c r="F51" s="303" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="G51" s="303" t="str">
-        <x:v>第十轮：当前仅持有管理员既有会话；新管理端登录使用所提供口令被拒绝，其他角色/首次改密账号无可用登录。不能以管理员代替多角色、撤权或首次改密页面验收。</x:v>
+        <x:v>第十二轮：隔离 PostgreSQL/PostGIS 中构造范围内、边界上、范围外目标；受限账号只见授权单位/区域的3个目标，选择空域后仅内点与边界2个，清空恢复3个。交叉单位/区域的同坐标目标列表不出现、详情404；前端平面算法与ST_Covers/ST_Touches一致。仅验证平面筛选与范围授权，不把位置关系当作违规结论。</x:v>
       </x:c>
       <x:c r="H51" s="303" t="str">
         <x:v>Codex</x:v>
@@ -23341,11 +23665,9 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J51" s="303" t="str">
-        <x:v>本轮报告；隔离回归日志；既有第八/九轮证据保留</x:v>
-      </x:c>
-      <x:c r="K51" s="303" t="str">
-        <x:v>前置条件未齐</x:v>
-      </x:c>
+        <x:v>qa-r12/main46-browser-corrected.log; main46-geometry-agreement.json; main46-all-ui.txt; main46-selected-ui.txt; main46-cleared-ui.txt; main46-selected.png</x:v>
+      </x:c>
+      <x:c r="K51" s="303" t="str"/>
     </x:row>
     <x:row r="52" ht="160" customHeight="1">
       <x:c r="A52" s="160">
@@ -23367,7 +23689,7 @@
         <x:v>暂时测不了</x:v>
       </x:c>
       <x:c r="G52" s="303" t="str">
-        <x:v>第十轮：缺同批次持续风险和已解除历史风险成对样本；现有状态不人工改写。</x:v>
+        <x:v>第十二轮：隔离PostGIS同批样本：已通知NOTIFIED风险仍显示红色异常光晕，已排除EXCLUDED不带map-alarm-active；范围筛选后2条、清空3条。不把已排除替代真实风险解除，现场解除的业务来源契约仍缺。</x:v>
       </x:c>
       <x:c r="H52" s="303" t="str">
         <x:v>Codex</x:v>
@@ -23376,7 +23698,7 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J52" s="303" t="str">
-        <x:v>第十轮报告；本轮回放/页面/隔离回归证据</x:v>
+        <x:v>qa-r12/main47-risk-marker-dom.json; main46-risk-selected.png; main46-risk-browser-final.log</x:v>
       </x:c>
       <x:c r="K52" s="303" t="str">
         <x:v>场景或环境前置条件未齐</x:v>
@@ -23432,10 +23754,10 @@
         <x:v>223</x:v>
       </x:c>
       <x:c r="F54" s="303" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="G54" s="303" t="str">
-        <x:v>第十轮：缺与本事件对应的可控反制/干扰/光电测试设备及可信最终回执；MQTT工参只证明连接和工作状态，健康UNKNOWN不能当GOOD，不能伪造实机收令或停机核查。</x:v>
+        <x:v>第十二轮：隔离页面已验证无位置提示不能引导光电、无权限提示无法读取、忙设备提示没有可用空闲设备；三种情况均无开始跟踪入口。仅气象无目标风险不显示光电跟踪、不造目标。28项API回归+1浏览器夹具通过，结束时跟踪任务和设备指令数量均未增加。</x:v>
       </x:c>
       <x:c r="H54" s="303" t="str">
         <x:v>Codex</x:v>
@@ -23444,11 +23766,9 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J54" s="303" t="str">
-        <x:v>本轮报告；隔离回归日志；既有第八/九轮证据保留</x:v>
-      </x:c>
-      <x:c r="K54" s="303" t="str">
-        <x:v>前置条件未齐</x:v>
-      </x:c>
+        <x:v>qa-r12/main49-api-guards-final.log; main49-browser.log; main49-no-permission-ui.txt; main49-missing-ui.txt; main49-busy-ui.txt; main49-weather-ui.txt; main49-busy.png</x:v>
+      </x:c>
+      <x:c r="K54" s="303" t="str"/>
     </x:row>
     <x:row r="55" ht="160" customHeight="1">
       <x:c r="A55" s="160">
@@ -23838,10 +24158,10 @@
         <x:v>253</x:v>
       </x:c>
       <x:c r="F66" s="303" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="G66" s="303" t="str">
-        <x:v>第十轮：当前取消现场观察写入按基线生效；尚缺本业务库可定位的旧现场冻结记录供页面只读对照。</x:v>
+        <x:v>第十二轮：告警详情恢复只读折叠历史，冻结材料保留原观察、紧急标记和办理人，明确不作为当前依据；切换事件不残留，三个视口无溢出。H2/PG历史及停用接口44项通过，实际页面夹具1项通过。</x:v>
       </x:c>
       <x:c r="H66" s="303" t="str">
         <x:v>Codex</x:v>
@@ -23850,11 +24170,9 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J66" s="303" t="str">
-        <x:v>第十轮报告；本轮回放/页面/隔离回归证据</x:v>
-      </x:c>
-      <x:c r="K66" s="303" t="str">
-        <x:v>场景或环境前置条件未齐</x:v>
-      </x:c>
+        <x:v>qa-r12/main61-history-regression.log; main61-browser-fixture-final.log; main61-alarm-ui.txt; main61-frozen-ui.txt; main61-switched-ui.txt; fix59-viewports.json; main61-alarm.png</x:v>
+      </x:c>
+      <x:c r="K66" s="303" t="str"/>
     </x:row>
     <x:row r="67" ht="160" customHeight="1">
       <x:c r="A67" s="178">
@@ -24317,7 +24635,7 @@
         <x:v>暂时测不了</x:v>
       </x:c>
       <x:c r="G80" s="303" t="str">
-        <x:v>第十轮：当前QA短信/电话未启用，且缺本批次核验飞手和完整送达/播放/持续位置链；现有隔离回归通过，但不能当作现场通知闭环。</x:v>
+        <x:v>第十二轮：新增短信、电话独立批次迟到回执回归：渠道执行中第二worker不重复发送，租约过期先落UNKNOWN，原成功回执迟到不能覆盖UNKNOWN、增加事件版本或新增联系记录；H2/PG均通过。完整页面多种重复/乱序组合仍未执行，浏览器当前连接不可用。</x:v>
       </x:c>
       <x:c r="H80" s="303" t="str">
         <x:v>Codex</x:v>
@@ -24326,7 +24644,7 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J80" s="303" t="str">
-        <x:v>本轮报告；隔离回归日志；既有第八/九轮证据保留</x:v>
+        <x:v>qa-r12/fix61-package-final.log; AutoSmsApiTest; AutoVoiceApiTest; browser-unavailable-1909.json</x:v>
       </x:c>
       <x:c r="K80" s="303" t="str">
         <x:v>前置条件未齐</x:v>
@@ -24726,10 +25044,10 @@
         <x:v>309</x:v>
       </x:c>
       <x:c r="F92" s="303" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="G92" s="303" t="str">
-        <x:v>第十二轮：已核实新旧事件不混用研判，旧事件409；位置过期页面阻断。隔离资格回归通过。</x:v>
+        <x:v>第十二轮：过期位置、合法、未知、证据不足、其他事件研判×申请/直接/执行三入口，H2与PostgreSQL共30项通过；追加新研判保留历史。隔离运行服务五种执行页面均明确本次没有下发，结束后5条授权仍APPROVED、EXECUTE事件0、设备指令0；未使用人工现场记录补资格。</x:v>
       </x:c>
       <x:c r="H92" s="303" t="str">
         <x:v>Codex</x:v>
@@ -24738,11 +25056,9 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J92" s="303" t="str">
-        <x:v>qa-r12/counter-r20/stop-race-green-package.log; counter-r20/concurrent-direct.json; counter-boundaries-tests.log</x:v>
-      </x:c>
-      <x:c r="K92" s="303" t="str">
-        <x:v>剩余：合法、未知、证据不足三类在申请/直接/执行入口的完整运行组合。</x:v>
-      </x:c>
+        <x:v>qa-r12/main87-entry-matrix-final.log;main87-browser-frozen-clock.log;main87-manifest.json;main87-STALE.png;main87-LEGAL.png;main87-UNKNOWN.png;main87-INSUFFICIENT.png;main87-OTHER_EVENT.png</x:v>
+      </x:c>
+      <x:c r="K92" s="303" t="str"/>
     </x:row>
     <x:row r="93" ht="160" customHeight="1">
       <x:c r="A93" s="192">
@@ -24761,10 +25077,10 @@
         <x:v>311</x:v>
       </x:c>
       <x:c r="F93" s="303" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="G93" s="303" t="str">
-        <x:v>第十二轮：DIRECT队列发令时重查身份、显式OP、数据范围、设备权限与窗口的隔离回归通过。</x:v>
+        <x:v>第十二轮：经正常DIRECT API创建实际QUEUED四通道指令后，分别撤DIRECT/设备权限、停用用户/角色、撤范围、授权过期、观测超过当前配置窗口；H2/PG各7项均CANCELLED，重复dispatch无issued_at、无回执、仍仅一条命令。另覆盖普通审批排队过期。仅隔离软件队列验收，不代表现场设备验收。</x:v>
       </x:c>
       <x:c r="H93" s="303" t="str">
         <x:v>Codex</x:v>
@@ -24773,10 +25089,10 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J93" s="303" t="str">
-        <x:v>qa-r12/counter-r20/stop-race-green-package.log; counter-r20/concurrent-direct.json; counter-boundaries-tests.log</x:v>
+        <x:v>qa-r12/direct-queued-eligibility-final.log;fix51-queue-final.log</x:v>
       </x:c>
       <x:c r="K93" s="303" t="str">
-        <x:v>剩余：实际运行服务排队后撤权/观测过期的不下发协议证据。</x:v>
+        <x:v>原有普通审批窗口缺陷FIX51已修复</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="160" customHeight="1">
@@ -24796,10 +25112,10 @@
         <x:v>313</x:v>
       </x:c>
       <x:c r="F94" s="303" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="G94" s="303" t="str">
-        <x:v>第十二轮：本机实际COUNTER→JAMMING续链已验证真实发起人与原窗口；撤权及到期隔离回归通过。</x:v>
+        <x:v>第十二轮：实际回环MQTT与正式授权流程在H2/PG覆盖正常、撤直接权限、撤设备权限、撤范围和原授权到期。正常收到60003与60002两命令，子授权DIRECT、真实原发起人、无审批人、截止沿用原窗口；四阻断分支原命令COMPLETED但无子授权、实收仅1条。到期分支补新有效观测与研判，单独断言依据仍有效，排除观测过期误阻断。重复结算不重发。</x:v>
       </x:c>
       <x:c r="H94" s="303" t="str">
         <x:v>Codex</x:v>
@@ -24808,11 +25124,9 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J94" s="303" t="str">
-        <x:v>qa-r12/counter-r20/stop-race-green-package.log; counter-r20/concurrent-direct.json; counter-boundaries-tests.log</x:v>
-      </x:c>
-      <x:c r="K94" s="303" t="str">
-        <x:v>剩余：实际服务续链间隙撤权/到期的协议不下发验证。</x:v>
-      </x:c>
+        <x:v>qa-r12/counter-r20/stop-race-green-package.log; counter-r20/concurrent-direct.json; counter-boundaries-tests.log;fix51-red.log;fix51-green.log;fix51-queue-final.log;main89-91-wire-final.log;main89-91-wire/h2/;main89-91-wire/postgresql/</x:v>
+      </x:c>
+      <x:c r="K94" s="303" t="str"/>
     </x:row>
     <x:row r="95" ht="160" customHeight="1">
       <x:c r="A95" s="192">
@@ -24831,10 +25145,10 @@
         <x:v>315</x:v>
       </x:c>
       <x:c r="F95" s="303" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="G95" s="303" t="str">
-        <x:v>第十二轮：同事件重复直接发起409；两请求并发仅一条201。旧设备待现场停机核查阻断且不走人工执行。</x:v>
+        <x:v>第十二轮：本机模拟完整覆盖占用、离线、故障：页面分别说明具体受阻，不走人工填写成功；H2/PG三种活动指令状态阻止第二事件启动，两账号两事件真实PG并发仅1启动。停用/离线无指令，排队变更取消且无发送时刻/回执；同事件重复与并发沿用已核验证据。停止/全关仍可排队。</x:v>
       </x:c>
       <x:c r="H95" s="303" t="str">
         <x:v>Codex</x:v>
@@ -24843,11 +25157,9 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J95" s="303" t="str">
-        <x:v>qa-r12/counter-r20/stop-race-green-package.log; counter-r20/concurrent-direct.json; counter-boundaries-tests.log</x:v>
-      </x:c>
-      <x:c r="K95" s="303" t="str">
-        <x:v>剩余：忙、离线、故障三组完整页面与指令历史组合。</x:v>
-      </x:c>
+        <x:v>qa-r12/counter-r20/stop-race-green-package.log; counter-r20/concurrent-direct.json; counter-boundaries-tests.log; fix52-53-final.log; fix52-fault-ui.png; fix52-fault-viewports.json; fix54-green.log; fix54-busy-ui.png; main90-offline-final.log; main90-offline-ui.png</x:v>
+      </x:c>
+      <x:c r="K95" s="303" t="str"/>
     </x:row>
     <x:row r="96" ht="160" customHeight="1">
       <x:c r="A96" s="192">
@@ -24866,10 +25178,10 @@
         <x:v>317</x:v>
       </x:c>
       <x:c r="F96" s="303" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="G96" s="303" t="str">
-        <x:v>第十二轮：真实TCP收令后4秒迟到回码：3秒时ADAPTER_TIMEOUT且成功回执0；同键重放原commandId，实际日志仅一次收令。协议无命令号，已关闭连接迟到帧不串到新任务、不补造原任务成功。</x:v>
+        <x:v>第十二轮：无命令号CM4迟到不串任务/不重发已验。带msgNo凌云在H2/PG真实MQTT迟到成功失败归原任务，并发去重，不覆盖超时/取消或新命令；普通审批实际页面下发后仅1条60003，3秒超时，50秒后迟到成功保留FAILED与原历史且不续链。页面明确超时不代表未执行，从原授权精确查看原命令，返回仍失败、无执行入口。</x:v>
       </x:c>
       <x:c r="H96" s="303" t="str">
         <x:v>Codex</x:v>
@@ -24878,11 +25190,9 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J96" s="303" t="str">
-        <x:v>qa-r12/counter-r22/late-reply.json; counter-r22/cm4.log; counter-reply-final-package.log</x:v>
-      </x:c>
-      <x:c r="K96" s="303" t="str">
-        <x:v>剩余：带命令关联号协议的迟到结果归属与普通反制执行页面全链；本机CM4迟到不重发已验。</x:v>
-      </x:c>
+        <x:v>qa-r12/counter-r22/late-reply.json; counter-r22/cm4.log; counter-reply-final-package.log;fix56-red.log;fix56-regression-package.log;fix56-regression-package-final.log;fix56-browser-checks.json;fix56-final.png;fix56-viewports.json;main89-91-wire-final.log;main91-before-late.json;fix57-timeout-ui.txt;main91-late-linked-ui.txt;main91-late-linked.png;main91-late-authorization-unchanged.txt;fix57-viewports.json;main91-browser-fixture.log</x:v>
+      </x:c>
+      <x:c r="K96" s="303" t="str"/>
     </x:row>
     <x:row r="97" ht="160" customHeight="1">
       <x:c r="A97" s="192">
@@ -25068,10 +25378,10 @@
         <x:v>329</x:v>
       </x:c>
       <x:c r="F102" s="303" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="G102" s="303" t="str">
-        <x:v>第十二轮：PostgreSQL真实锁竞争和同键并发通过；运行服务设备收令等待回码时急停200且无重复命令。</x:v>
+        <x:v>第十二轮：PG两起点三方并发及同键重放通过；独立运行服务三账号实际HTTP竞态分别形成EXECUTING/1命令和CANCELLED/0命令。第三请求确认等待PG事件锁时强制终止进程，数据库事务无新增；原库新进程重启后6个旧请求409，中断请求同键200且仅1命令，再重放409。办理历史与实际成功操作一致。</x:v>
       </x:c>
       <x:c r="H102" s="303" t="str">
         <x:v>Codex</x:v>
@@ -25080,11 +25390,9 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J102" s="303" t="str">
-        <x:v>qa-r12/counter-r20/stop-race-green-package.log; counter-r20/concurrent-direct.json; counter-boundaries-tests.log</x:v>
-      </x:c>
-      <x:c r="K102" s="303" t="str">
-        <x:v>剩余：批准/撤销/执行三方并发及短时重启组合。</x:v>
-      </x:c>
+        <x:v>qa-r12/main87-97-105-regression.log;main97-http-races.json;main97-interrupted-http.json;main97-before-crash.json;main97-after-crash.json;main97-restart-replays.json;main97-after-replays.json;main97-summary.json;main97-process-restored.log</x:v>
+      </x:c>
+      <x:c r="K102" s="303" t="str"/>
     </x:row>
     <x:row r="103" ht="160" customHeight="1">
       <x:c r="A103" s="195">
@@ -25340,10 +25648,10 @@
         <x:v>345</x:v>
       </x:c>
       <x:c r="F110" s="303" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="G110" s="303" t="str">
-        <x:v>第十二轮：真实模拟交接后续续配通道、失败补发、迟到回执与签收均不改变冻结材料和原接收快照。新证据追加及DIRECT真实发起人组合仍待补，不提升完整状态。</x:v>
+        <x:v>第十二轮：H2/PG正式接口直接发起→停止授权→上传关联真实测试日志→移送→后补日志；旧快照全文不变，DIRECT保留原发起人且无审批人，后补证据仅追加事件关联。页面补显示冻结发起人与移送时证据，和当前关联证据分开；改名不改旧材料，精确链接打开before.txt，普通审批记录保留审批人。</x:v>
       </x:c>
       <x:c r="H110" s="303" t="str">
         <x:v>Codex</x:v>
@@ -25352,11 +25660,9 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J110" s="303" t="str">
-        <x:v>qa-r12/handoff-material-before.json; handoff-receipt-invariants.json</x:v>
-      </x:c>
-      <x:c r="K110" s="303" t="str">
-        <x:v>前置条件未齐</x:v>
-      </x:c>
+        <x:v>qa-r12/main105-direct-frozen.log;main87-97-105-regression.log;fix55-before-ui.txt;fix55-after-ui.txt;fix55-final.png;fix55-viewports.json;fix55-frozen-link-ui.txt;fix55-ordinary-ui.txt;fix55-build-final.log;fix55-scan.log</x:v>
+      </x:c>
+      <x:c r="K110" s="303" t="str"/>
     </x:row>
     <x:row r="111" ht="160" customHeight="1">
       <x:c r="A111" s="201">
@@ -25822,10 +26128,10 @@
         <x:v>382</x:v>
       </x:c>
       <x:c r="F124" s="303" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="G124" s="303" t="str">
-        <x:v>第十轮：缺统计边界前后独立观测/案件样本；现有日期筛选与导出一致，不替代边界真值。</x:v>
+        <x:v>第十二轮：隔离H2/PostgreSQL对开始前1ms、开始零点、结束日末1ms、次日零点六组目标/立案时间逐项验证。26回归通过；独立PostGIS浏览器实际两单日2/0、2/1及跨年两日4/1均正确，重复末次观测未新增计数；CSV接口200且总数4。仅使用一次性合成统计事实，不证明真实处罚结果；浏览器下载连接中断未另算下载通过。</x:v>
       </x:c>
       <x:c r="H124" s="303" t="str">
         <x:v>Codex</x:v>
@@ -25834,11 +26140,9 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J124" s="303" t="str">
-        <x:v>第十轮报告；本轮回放/页面/隔离回归证据</x:v>
-      </x:c>
-      <x:c r="K124" s="303" t="str">
-        <x:v>场景或环境前置条件未齐</x:v>
-      </x:c>
+        <x:v>qa-r12/main119-api.log; main119-browser-final.log; main119-manifest.json; main119-api-facts.json; main119-day1-ui.txt; main119-day2-ui.txt; main119-range-ui.txt; main119-api-export.csv</x:v>
+      </x:c>
+      <x:c r="K124" s="303" t="str"/>
     </x:row>
     <x:row r="125" ht="160" customHeight="1">
       <x:c r="A125" s="219">
@@ -26132,7 +26436,7 @@
         <x:v>暂时测不了</x:v>
       </x:c>
       <x:c r="G133" s="303" t="str">
-        <x:v>第十轮：键盘缩放组合未使实际CSS视口/像素比例变化，不能声称200%已验；需要能控制浏览器原生缩放的环境。</x:v>
+        <x:v>第十二轮：Edge键盘Tab/Shift+Tab、Enter走通导航、空域搜索、地图控件焦点、详情打开/关闭；焦点与文字状态有证据。浏览器缩放快捷键未改变可验证缩放，真实200%未验收，不把窗口尺寸代替缩放。</x:v>
       </x:c>
       <x:c r="H133" s="303" t="str">
         <x:v>Codex</x:v>
@@ -26141,7 +26445,7 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J133" s="303" t="str">
-        <x:v>视口观察记录</x:v>
+        <x:v>qa-r12/main128-focus-walk.json; main128-keyboard-search.txt; main128-keyboard-search.png</x:v>
       </x:c>
       <x:c r="K133" s="303" t="str">
         <x:v>200%缩放尚未生效</x:v>
@@ -26202,7 +26506,7 @@
         <x:v>暂时测不了</x:v>
       </x:c>
       <x:c r="G135" s="303" t="str">
-        <x:v>第十轮：Edge已完成关键路径；当前自动化连接仅Edge和内置浏览器，没有可控Chrome连接，未将Edge结果冒充Chrome。</x:v>
+        <x:v>第十二轮：已连接Edge 154.0.4258.37，本轮登录、表单、地图及视频状态流程有实测。当前CUA仅提供Edge与内置浏览器，未连接Chrome；两浏览器完整对照仍未完成。</x:v>
       </x:c>
       <x:c r="H135" s="303" t="str">
         <x:v>Codex</x:v>
@@ -26211,7 +26515,7 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J135" s="303" t="str">
-        <x:v>浏览器可用连接清单</x:v>
+        <x:v>qa-r12/main130-browser-environment.json</x:v>
       </x:c>
       <x:c r="K135" s="303" t="str">
         <x:v>需Chrome连接</x:v>
@@ -26710,10 +27014,10 @@
         <x:v>444</x:v>
       </x:c>
       <x:c r="F150" s="303" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="G150" s="303" t="str">
-        <x:v>第十轮：当前仅持有管理员既有会话；新管理端登录使用所提供口令被拒绝，其他角色/首次改密账号无可用登录。不能以管理员代替多角色、撤权或首次改密页面验收。</x:v>
+        <x:v>第十二轮：隔离PostGIS构造两个单位同名空域，甲单位含mock/replay/live三种来源。甲账号只见本单位3条且逐条打开编号正确；退出换乙账号只见乙单位1条，旧列表/详情不残留。模拟/回放独立标记，源模式API一致；双方访问另一单位详情均404。</x:v>
       </x:c>
       <x:c r="H150" s="303" t="str">
         <x:v>Codex</x:v>
@@ -26722,11 +27026,9 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J150" s="303" t="str">
-        <x:v>本轮报告；隔离回归日志；既有第八/九轮证据保留</x:v>
-      </x:c>
-      <x:c r="K150" s="303" t="str">
-        <x:v>前置条件未齐</x:v>
-      </x:c>
+        <x:v>qa-r12/main145-browser-final.log; main145-manifest.json; main145-account-a-ui.txt; main145-a-details.json; main145-account-b-ui.txt; main145-b-detail.txt; main145-account-a.png; main145-account-b.png</x:v>
+      </x:c>
+      <x:c r="K150" s="303" t="str"/>
     </x:row>
     <x:row r="151" ht="160" customHeight="1">
       <x:c r="A151" s="240">
@@ -26816,7 +27118,7 @@
         <x:v>暂时测不了</x:v>
       </x:c>
       <x:c r="G153" s="303" t="str">
-        <x:v>第十轮：缺本组合独立规则版本、已核验主体和可执行设备回执链；自动服务隔离测试已通过，但未将单个条件分支扩记为自动/手动整链通过。</x:v>
+        <x:v>第十二轮：真实AutomationRuntimeWorker与持久化服务在H2/PG完成事实源异常→错误心跳→恢复→仅核实一次；新建worker实例再次轮询无重复核实/运行记录。事实输入受控模拟，尚未覆盖独立JVM启动故障与重启后的全部外发动作，不能将bean重建冒报进程重启验收。</x:v>
       </x:c>
       <x:c r="H153" s="303" t="str">
         <x:v>Codex</x:v>
@@ -26825,7 +27127,7 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J153" s="303" t="str">
-        <x:v>本轮报告；隔离回归日志；既有第八/九轮证据保留</x:v>
+        <x:v>qa-r12/fix61-package-final.log; fix61-worker-pg.log; AlarmRuleVerificationTest</x:v>
       </x:c>
       <x:c r="K153" s="303" t="str">
         <x:v>前置条件未齐</x:v>
@@ -26921,7 +27223,7 @@
         <x:v>暂时测不了</x:v>
       </x:c>
       <x:c r="G156" s="303" t="str">
-        <x:v>第十轮：缺本组合独立规则版本、已核验主体和可执行设备回执链；自动服务隔离测试已通过，但未将单个条件分支扩记为自动/手动整链通过。</x:v>
+        <x:v>第十二轮：FIX60已复现并修复自动主体排队/续链绕过引擎关闭的问题；当前引擎、规则版本/时段及事实重新核对。H2/PG资格、实际MQTT普通/直接续链和认证等248测试通过，2个opt-in跳过。仍需自动规则实际启动到规则修改的同批完整运行组合，未将守卫回归当全链通过。 FIX61进一步修复自动核实/反制入口沿用旧PASS：事件/类别/当前判定记录及当前规则再核对，设备锁后再查。</x:v>
       </x:c>
       <x:c r="H156" s="303" t="str">
         <x:v>Codex</x:v>
@@ -26930,7 +27232,7 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J156" s="303" t="str">
-        <x:v>本轮报告；隔离回归日志；既有第八/九轮证据保留</x:v>
+        <x:v>qa-r12/fix60-red.log; fix60-green.log; fix60-package.log; fix60-services.json; fix61-red.log; fix61-green.log; fix61-package-final.log; fix61-worker-pg.log</x:v>
       </x:c>
       <x:c r="K156" s="303" t="str">
         <x:v>前置条件未齐</x:v>
@@ -27001,7 +27303,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cdc5136b2714173"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff207c4ba6a247a2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29880,7 +30182,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67432706291e4856"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd716ef1bf2cc46c1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31271,22 +31573,21 @@
       <x:c r="E31" s="91" t="s">
         <x:v>1151</x:v>
       </x:c>
-      <x:c r="F31" s="44" t="s">
-        <x:v>1061</x:v>
+      <x:c r="F31" s="44" t="str">
+        <x:v>R12-PG-F26-bd862e03（隔离模拟）</x:v>
       </x:c>
       <x:c r="G31" s="44" t="str">
         <x:f>IF(COUNTIF('流程步骤记录'!G256:G265,"有问题")&gt;0,"有问题",IF(COUNTIF('流程步骤记录'!G256:G265,"暂时测不了")&gt;0,"暂时测不了",IF(COUNTBLANK('流程步骤记录'!G256:G265)&gt;0,"未填结果",IF(COUNTIF('流程步骤记录'!G256:G265,"通过")=10,IF(COUNTBLANK('流程步骤记录'!H256:L265)&gt;0,"待补证据","通过"),IF(COUNTIF('流程步骤记录'!G256:G265,"还没测")=10,"还没测","进行中")))))</x:f>
         <x:v>暂时测不了</x:v>
       </x:c>
-      <x:c r="H31" s="44" t="s">
-        <x:v>92</x:v>
+      <x:c r="H31" s="44" t="str">
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="I31" s="45" t="str">
-        <x:v>第十轮</x:v>
+        <x:v>第十二轮</x:v>
       </x:c>
       <x:c r="J31" s="44" t="str">
-        <x:v>第十轮：尚未完成同一批次全部十步；浏览器阻塞已解除。当前场景：计划到时未发现目标，测试设备异常检查及通知后台；后台处理后分别验证恢复成功和未恢复。。局部修复与回归见本轮报告。历史前置记录（需按现状回读，不是本轮通过）：第八轮：未完成整项。缺独立健康GOOD的恢复样本或所需TCP/光电协议测试回执；MQTT在线和UNKNOWN不能冒充健康恢复。
-证据：第八轮报告；r8-current-preconditions.json；r8-frozen-final-summary.json</x:v>
+        <x:v>逐步证据见流程步骤记录，隔离模拟批次</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="180" customHeight="1">
@@ -31305,22 +31606,21 @@
       <x:c r="E32" s="23" t="s">
         <x:v>1156</x:v>
       </x:c>
-      <x:c r="F32" s="20" t="s">
-        <x:v>1061</x:v>
+      <x:c r="F32" s="20" t="str">
+        <x:v>R12-MQTT-BIRD-B-703e2e19</x:v>
       </x:c>
       <x:c r="G32" s="20" t="str">
         <x:f>IF(COUNTIF('流程步骤记录'!G266:G275,"有问题")&gt;0,"有问题",IF(COUNTIF('流程步骤记录'!G266:G275,"暂时测不了")&gt;0,"暂时测不了",IF(COUNTBLANK('流程步骤记录'!G266:G275)&gt;0,"未填结果",IF(COUNTIF('流程步骤记录'!G266:G275,"通过")=10,IF(COUNTBLANK('流程步骤记录'!H266:L275)&gt;0,"待补证据","通过"),IF(COUNTIF('流程步骤记录'!G266:G275,"还没测")=10,"还没测","进行中")))))</x:f>
         <x:v>暂时测不了</x:v>
       </x:c>
-      <x:c r="H32" s="20" t="s">
-        <x:v>92</x:v>
+      <x:c r="H32" s="20" t="str">
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="I32" s="21" t="str">
-        <x:v>第十轮</x:v>
+        <x:v>第十二轮</x:v>
       </x:c>
       <x:c r="J32" s="20" t="str">
-        <x:v>第十轮：尚未完成同一批次全部十步；浏览器阻塞已解除。当前场景：用同一鸟群从发现走到通知、反馈和风险解除；不进入无人机合法性或反制链。。局部修复与回归见本轮报告。历史前置记录（需按现状回读，不是本轮通过）：第八轮部分验证，整项未完成：同一鸟类批次已完成发现、风险生成、核验和通知交接，未进无人机研判；配置未启用阻断实际投递，反馈/解除闭环未完成。
-证据：r8-bird-evaluation.json；r8-risk-verification.json；r8-risk-final.json</x:v>
+        <x:v>逐步证据见流程步骤记录，隔离模拟批次</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="180" customHeight="1">
@@ -31441,22 +31741,21 @@
       <x:c r="E36" s="5" t="s">
         <x:v>1175</x:v>
       </x:c>
-      <x:c r="F36" s="20" t="s">
-        <x:v>1061</x:v>
+      <x:c r="F36" s="20" t="str">
+        <x:v>R12-PG-F31-ce4e5b9b（隔离协议模拟）</x:v>
       </x:c>
       <x:c r="G36" s="20" t="str">
         <x:f>IF(COUNTIF('流程步骤记录'!G306:G315,"有问题")&gt;0,"有问题",IF(COUNTIF('流程步骤记录'!G306:G315,"暂时测不了")&gt;0,"暂时测不了",IF(COUNTBLANK('流程步骤记录'!G306:G315)&gt;0,"未填结果",IF(COUNTIF('流程步骤记录'!G306:G315,"通过")=10,IF(COUNTBLANK('流程步骤记录'!H306:L315)&gt;0,"待补证据","通过"),IF(COUNTIF('流程步骤记录'!G306:G315,"还没测")=10,"还没测","进行中")))))</x:f>
         <x:v>暂时测不了</x:v>
       </x:c>
-      <x:c r="H36" s="20" t="s">
-        <x:v>92</x:v>
+      <x:c r="H36" s="20" t="str">
+        <x:v>Codex</x:v>
       </x:c>
       <x:c r="I36" s="21" t="str">
-        <x:v>第十轮</x:v>
+        <x:v>第十二轮</x:v>
       </x:c>
       <x:c r="J36" s="20" t="str">
-        <x:v>第十轮：尚未完成同一批次全部十步；浏览器阻塞已解除。当前场景：登记测试雷达，完成调测并发送目标，核对前后台同源。。局部修复与回归见本轮报告。历史前置记录（需按现状回读，不是本轮通过）：第八轮：未完成整项。缺独立健康GOOD的恢复样本或所需TCP/光电协议测试回执；MQTT在线和UNKNOWN不能冒充健康恢复。
-证据：第八轮报告；r8-current-preconditions.json；r8-frozen-final-summary.json</x:v>
+        <x:v>逐步证据见流程步骤记录，隔离模拟批次</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="180" customHeight="1">
@@ -31694,7 +31993,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0e38c90034b4f1c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R196f50521ee149c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -41329,22 +41628,22 @@
         <x:v>1384</x:v>
       </x:c>
       <x:c r="G256" s="48" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H256" s="48" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：准备已到计划起飞时间但未收到目标的计划；设备异常、正常、信息不足三个子批次。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮：未完成整项。缺独立健康GOOD的恢复样本或所需TCP/光电协议测试回执；MQTT在线和UNKNOWN不能冒充健康恢复。</x:v>
-      </x:c>
-      <x:c r="I256" s="48" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J256" s="49">
-        <x:v>46293</x:v>
+        <x:v>独立PG库qa0929r12f，同计划seed-stage3-plan-legal/设备0d2e49c7/任务bd862e03；正常、BAD、UNKNOWN使用不同场景指令ID。</x:v>
+      </x:c>
+      <x:c r="I256" s="48" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J256" s="328" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K256" s="48" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L256" s="48" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/f26/；f26-pg-fixture-final.log</x:v>
+      </x:c>
+      <x:c r="L256" s="48" t="str">
+        <x:v>R12-PG-F26-bd862e03（隔离模拟）</x:v>
       </x:c>
     </x:row>
     <x:row r="257" ht="160" customHeight="1">
@@ -41367,22 +41666,22 @@
         <x:v>1387</x:v>
       </x:c>
       <x:c r="G257" s="44" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H257" s="44" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：打开飞行计划检查结果和最近观测。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮：未完成整项。缺独立健康GOOD的恢复样本或所需TCP/光电协议测试回执；MQTT在线和UNKNOWN不能冒充健康恢复。</x:v>
-      </x:c>
-      <x:c r="I257" s="44" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J257" s="45">
-        <x:v>46293</x:v>
+        <x:v>前台明确未找到对应飞机，不据此断言没有起飞；计划处于到时执行窗口。</x:v>
+      </x:c>
+      <x:c r="I257" s="44" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J257" s="329" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K257" s="44" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L257" s="44" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/f26/；f26-pg-fixture-final.log</x:v>
+      </x:c>
+      <x:c r="L257" s="44" t="str">
+        <x:v>R12-PG-F26-bd862e03（隔离模拟）</x:v>
       </x:c>
     </x:row>
     <x:row r="258" ht="160" customHeight="1">
@@ -41405,22 +41704,22 @@
         <x:v>1390</x:v>
       </x:c>
       <x:c r="G258" s="44" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H258" s="44" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：按已有规则读取设备检查；对照实际设备异常及最近上报。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮：未完成整项。缺独立健康GOOD的恢复样本或所需TCP/光电协议测试回执；MQTT在线和UNKNOWN不能冒充健康恢复。</x:v>
-      </x:c>
-      <x:c r="I258" s="44" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J258" s="45">
-        <x:v>46293</x:v>
+        <x:v>同一设备0米范围：GOOD疑似未起飞、BAD自动设备异常、UNKNOWN检查不完整，API与页面一致。</x:v>
+      </x:c>
+      <x:c r="I258" s="44" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J258" s="329" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K258" s="44" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L258" s="44" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/f26/；f26-pg-fixture-final.log</x:v>
+      </x:c>
+      <x:c r="L258" s="44" t="str">
+        <x:v>R12-PG-F26-bd862e03（隔离模拟）</x:v>
       </x:c>
     </x:row>
     <x:row r="259" ht="160" customHeight="1">
@@ -41443,22 +41742,22 @@
         <x:v>1393</x:v>
       </x:c>
       <x:c r="G259" s="44" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H259" s="44" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：对实际异常用有权账号通知，重复点击并记录操作结果。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮：未完成整项。缺独立健康GOOD的恢复样本或所需TCP/光电协议测试回执；MQTT在线和UNKNOWN不能冒充健康恢复。</x:v>
-      </x:c>
-      <x:c r="I259" s="44" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J259" s="45">
-        <x:v>46293</x:v>
+        <x:v>正常API同键及异键三次重复通知均复用bd862e03，通知仍1；审计只读账号403。</x:v>
+      </x:c>
+      <x:c r="I259" s="44" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J259" s="329" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K259" s="44" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L259" s="44" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/f26/；f26-pg-fixture-final.log</x:v>
+      </x:c>
+      <x:c r="L259" s="44" t="str">
+        <x:v>R12-PG-F26-bd862e03（隔离模拟）</x:v>
       </x:c>
     </x:row>
     <x:row r="260" ht="160" customHeight="1">
@@ -41481,22 +41780,22 @@
         <x:v>1396</x:v>
       </x:c>
       <x:c r="G260" s="44" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H260" s="44" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：在管理后台找到前台产生的同一事项，核对设备、时间及异常原因。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮：未完成整项。缺独立健康GOOD的恢复样本或所需TCP/光电协议测试回执；MQTT在线和UNKNOWN不能冒充健康恢复。</x:v>
-      </x:c>
-      <x:c r="I260" s="44" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J260" s="45">
-        <x:v>46293</x:v>
+        <x:v>后台从运维消息进入同一bd862e03/DEV-MOCK-004/计划-0905-001，时间及异常快照一致。</x:v>
+      </x:c>
+      <x:c r="I260" s="44" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J260" s="329" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K260" s="44" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L260" s="44" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/f26/；f26-pg-fixture-final.log</x:v>
+      </x:c>
+      <x:c r="L260" s="44" t="str">
+        <x:v>R12-PG-F26-bd862e03（隔离模拟）</x:v>
       </x:c>
     </x:row>
     <x:row r="261" ht="160" customHeight="1">
@@ -41522,19 +41821,19 @@
         <x:v>暂时测不了</x:v>
       </x:c>
       <x:c r="H261" s="44" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：按已有流程处理测试设备异常；分别模拟处理成功、失败及回复未知。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮：未完成整项。缺独立健康GOOD的恢复样本或所需TCP/光电协议测试回执；MQTT在线和UNKNOWN不能冒充健康恢复。</x:v>
-      </x:c>
-      <x:c r="I261" s="44" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J261" s="45">
-        <x:v>46293</x:v>
+        <x:v>本批完成后台接手、提交核验、FAIL/UNKNOWN/PASS与完成全链；尚未补同一待办下真实协议设备命令成功/失败/迟到回复三个分支，不能把恢复核验结果当设备回执。</x:v>
+      </x:c>
+      <x:c r="I261" s="44" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J261" s="329" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K261" s="44" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L261" s="44" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/f26/；f26-pg-fixture-final.log</x:v>
+      </x:c>
+      <x:c r="L261" s="44" t="str">
+        <x:v>R12-PG-F26-bd862e03（隔离模拟）</x:v>
       </x:c>
     </x:row>
     <x:row r="262" ht="160" customHeight="1">
@@ -41557,22 +41856,22 @@
         <x:v>1402</x:v>
       </x:c>
       <x:c r="G262" s="44" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H262" s="44" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：恢复设备上报和健康数据；另一子批次仅完成后台处理但不恢复设备。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮：未完成整项。缺独立健康GOOD的恢复样本或所需TCP/光电协议测试回执；MQTT在线和UNKNOWN不能冒充健康恢复。</x:v>
-      </x:c>
-      <x:c r="I262" s="44" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J262" s="45">
-        <x:v>46293</x:v>
+        <x:v>BAD和UNKNOWN均保持待恢复核验且COMPLETE409；更新为新鲜GOOD/ONLINE无告警才PASS。明确模拟来源，不替代现场恢复。</x:v>
+      </x:c>
+      <x:c r="I262" s="44" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J262" s="329" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K262" s="44" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L262" s="44" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/f26/；f26-pg-fixture-final.log</x:v>
+      </x:c>
+      <x:c r="L262" s="44" t="str">
+        <x:v>R12-PG-F26-bd862e03（隔离模拟）</x:v>
       </x:c>
     </x:row>
     <x:row r="263" ht="160" customHeight="1">
@@ -41595,22 +41894,22 @@
         <x:v>1405</x:v>
       </x:c>
       <x:c r="G263" s="44" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H263" s="44" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：回到原计划和融合感知查看设备状态、异常提示及检查依据。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮：未完成整项。缺独立健康GOOD的恢复样本或所需TCP/光电协议测试回执；MQTT在线和UNKNOWN不能冒充健康恢复。</x:v>
-      </x:c>
-      <x:c r="I263" s="44" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J263" s="45">
-        <x:v>46293</x:v>
+        <x:v>原计划仍显示故障或未知直至对应状态改变；恢复后前台正常/待办已完成，融合感知同DEV-MOCK-004在线并保留模拟标识。</x:v>
+      </x:c>
+      <x:c r="I263" s="44" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J263" s="329" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K263" s="44" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L263" s="44" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/f26/；f26-pg-fixture-final.log</x:v>
+      </x:c>
+      <x:c r="L263" s="44" t="str">
+        <x:v>R12-PG-F26-bd862e03（隔离模拟）</x:v>
       </x:c>
     </x:row>
     <x:row r="264" ht="160" customHeight="1">
@@ -41633,22 +41932,22 @@
         <x:v>1408</x:v>
       </x:c>
       <x:c r="G264" s="44" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H264" s="44" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：核对计划未见目标提示、处理历史及异常通知记录。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮：未完成整项。缺独立健康GOOD的恢复样本或所需TCP/光电协议测试回执；MQTT在线和UNKNOWN不能冒充健康恢复。</x:v>
-      </x:c>
-      <x:c r="I264" s="44" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J264" s="45">
-        <x:v>46293</x:v>
+        <x:v>计划仍EXECUTING且未匹配飞机；原通知及接收快照逐字段不变，恢复历史保留FAIL/UNKNOWN/PASS，待办1、通知1。</x:v>
+      </x:c>
+      <x:c r="I264" s="44" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J264" s="329" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K264" s="44" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L264" s="44" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/f26/；f26-pg-fixture-final.log</x:v>
+      </x:c>
+      <x:c r="L264" s="44" t="str">
+        <x:v>R12-PG-F26-bd862e03（隔离模拟）</x:v>
       </x:c>
     </x:row>
     <x:row r="265" ht="160" customHeight="1">
@@ -41671,22 +41970,22 @@
         <x:v>1410</x:v>
       </x:c>
       <x:c r="G265" s="44" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H265" s="44" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：重新登录回查同一计划和设备；结束模拟并核对停止。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮：未完成整项。缺独立健康GOOD的恢复样本或所需TCP/光电协议测试回执；MQTT在线和UNKNOWN不能冒充健康恢复。</x:v>
-      </x:c>
-      <x:c r="I265" s="44" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J265" s="45">
-        <x:v>46293</x:v>
+        <x:v>前后台均退出后重新登录回查同一计划和任务；状态与六条办理历史一致，控制台error0，隔离输入STOP已确认。</x:v>
+      </x:c>
+      <x:c r="I265" s="44" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J265" s="329" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K265" s="44" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L265" s="44" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/f26/；f26-pg-fixture-final.log</x:v>
+      </x:c>
+      <x:c r="L265" s="44" t="str">
+        <x:v>R12-PG-F26-bd862e03（隔离模拟）</x:v>
       </x:c>
     </x:row>
     <x:row r="266" ht="160" customHeight="1">
@@ -41709,22 +42008,22 @@
         <x:v>1413</x:v>
       </x:c>
       <x:c r="G266" s="20" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H266" s="20" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：准备鸟群原始输入、重点区域、核验账号及模拟上级通道。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮部分验证，整项未完成：同一鸟类批次已完成发现、风险生成、核验和通知交接，未进无人机研判；配置未启用阻断实际投递，反馈/解除闭环未完成。</x:v>
-      </x:c>
-      <x:c r="I266" s="20" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J266" s="21">
-        <x:v>46293</x:v>
+        <x:v>本批原始 MQTT 雷达/TDOA 鸟群输入，planB 703e2e19、riskB a4d26a44 与 MOCK 上级通道有完整来源及范围。</x:v>
+      </x:c>
+      <x:c r="I266" s="20" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J266" s="302" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K266" s="20" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L266" s="20" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/bird-final-samples.json;bird-f27/b-accepted-history.json</x:v>
+      </x:c>
+      <x:c r="L266" s="20" t="str">
+        <x:v>R12-MQTT-BIRD-B-703e2e19</x:v>
       </x:c>
     </x:row>
     <x:row r="267" ht="160" customHeight="1">
@@ -41747,22 +42046,22 @@
         <x:v>1416</x:v>
       </x:c>
       <x:c r="G267" s="20" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H267" s="20" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：经真实测试接入发原始样本，记录平台统一目标。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮部分验证，整项未完成：同一鸟类批次已完成发现、风险生成、核验和通知交接，未进无人机研判；配置未启用阻断实际投递，反馈/解除闭环未完成。</x:v>
-      </x:c>
-      <x:c r="I267" s="20" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J267" s="21">
-        <x:v>46293</x:v>
+        <x:v>鸟群目标66fcf717由MQTT样本融合，source_links保留雷达87bd2b89与TDOA50ac45d1；未直接写风险结果。</x:v>
+      </x:c>
+      <x:c r="I267" s="20" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J267" s="302" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K267" s="20" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L267" s="20" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/bird-f27/history-target.json;bird-final-samples.json</x:v>
+      </x:c>
+      <x:c r="L267" s="20" t="str">
+        <x:v>R12-MQTT-BIRD-B-703e2e19</x:v>
       </x:c>
     </x:row>
     <x:row r="268" ht="160" customHeight="1">
@@ -41785,22 +42084,22 @@
         <x:v>1419</x:v>
       </x:c>
       <x:c r="G268" s="20" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H268" s="20" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：在空域或飞行计划全部风险中找到本次风险。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮部分验证，整项未完成：同一鸟类批次已完成发现、风险生成、核验和通知交接，未进无人机研判；配置未启用阻断实际投递，反馈/解除闭环未完成。</x:v>
-      </x:c>
-      <x:c r="I268" s="20" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J268" s="21">
-        <x:v>46293</x:v>
+        <x:v>飞行计划EXT-SIM-703e2e19进入风险-0929-002，鸟群、走廊内、距航线0米、60m AGL、发生时刻与风险接口一致。</x:v>
+      </x:c>
+      <x:c r="I268" s="20" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J268" s="302" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K268" s="20" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L268" s="20" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/bird-f27/accepted-history-ui.png;bird-f27/b-accepted-history.json</x:v>
+      </x:c>
+      <x:c r="L268" s="20" t="str">
+        <x:v>R12-MQTT-BIRD-B-703e2e19</x:v>
       </x:c>
     </x:row>
     <x:row r="269" ht="160" customHeight="1">
@@ -41823,22 +42122,22 @@
         <x:v>1422</x:v>
       </x:c>
       <x:c r="G269" s="20" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H269" s="20" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：查看合法性及无人机反制记录。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮部分验证，整项未完成：同一鸟类批次已完成发现、风险生成、核验和通知交接，未进无人机研判；配置未启用阻断实际投递，反馈/解除闭环未完成。</x:v>
-      </x:c>
-      <x:c r="I269" s="20" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J269" s="21">
-        <x:v>46293</x:v>
+        <x:v>该鸟群70条研判均NOT_APPLICABLE、无关联告警；UAV限定列表总数0。目标allowed_actions为空，未被认定黑飞。</x:v>
+      </x:c>
+      <x:c r="I269" s="20" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J269" s="302" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K269" s="20" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L269" s="20" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/bird-f27/branch-current.json;bird-f27/uav-filter.json</x:v>
+      </x:c>
+      <x:c r="L269" s="20" t="str">
+        <x:v>R12-MQTT-BIRD-B-703e2e19</x:v>
       </x:c>
     </x:row>
     <x:row r="270" ht="160" customHeight="1">
@@ -41861,22 +42160,22 @@
         <x:v>1425</x:v>
       </x:c>
       <x:c r="G270" s="20" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H270" s="20" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：有权账号在风险详情核验属实。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮部分验证，整项未完成：同一鸟类批次已完成发现、风险生成、核验和通知交接，未进无人机研判；配置未启用阻断实际投递，反馈/解除闭环未完成。</x:v>
-      </x:c>
-      <x:c r="I270" s="20" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J270" s="21">
-        <x:v>46293</x:v>
+        <x:v>同一风险人工CONFIRMED历史1条，保留核验人、时间及原始说明；通知页没有再次核验入口。</x:v>
+      </x:c>
+      <x:c r="I270" s="20" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J270" s="302" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K270" s="20" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L270" s="20" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/bird-f27/history-target.json;bird-f27/accepted-history-ui.png</x:v>
+      </x:c>
+      <x:c r="L270" s="20" t="str">
+        <x:v>R12-MQTT-BIRD-B-703e2e19</x:v>
       </x:c>
     </x:row>
     <x:row r="271" ht="160" customHeight="1">
@@ -41899,22 +42198,22 @@
         <x:v>1427</x:v>
       </x:c>
       <x:c r="G271" s="20" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H271" s="20" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：发送本风险通知并核对接收对象。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮部分验证，整项未完成：同一鸟类批次已完成发现、风险生成、核验和通知交接，未进无人机研判；配置未启用阻断实际投递，反馈/解除闭环未完成。</x:v>
-      </x:c>
-      <x:c r="I271" s="20" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J271" s="21">
-        <x:v>46293</x:v>
+        <x:v>同一通知d8da2cc9提交、送达、签收时间独立；接收快照上级、MOCK与原有效配置一致，页面显示已送达/已回执。</x:v>
+      </x:c>
+      <x:c r="I271" s="20" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J271" s="302" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K271" s="20" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L271" s="20" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/bird-f27/b-accepted-history.json;bird-f27/accepted-history-ui.png</x:v>
+      </x:c>
+      <x:c r="L271" s="20" t="str">
+        <x:v>R12-MQTT-BIRD-B-703e2e19</x:v>
       </x:c>
     </x:row>
     <x:row r="272" ht="160" customHeight="1">
@@ -41940,19 +42239,19 @@
         <x:v>暂时测不了</x:v>
       </x:c>
       <x:c r="H272" s="20" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：返回签收回执，同时保持鸟群有效观测。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮部分验证，整项未完成：同一鸟类批次已完成发现、风险生成、核验和通知交接，未进无人机研判；配置未启用阻断实际投递，反馈/解除闭环未完成。</x:v>
-      </x:c>
-      <x:c r="I272" s="20" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J272" s="21">
-        <x:v>46293</x:v>
+        <x:v>签收后风险保留UNKNOWN，未误解除。空间风险没有已确认的当前持续判定契约，无法证明有效观测时显示CURRENT，不把UNKNOWN当持续正向通过。</x:v>
+      </x:c>
+      <x:c r="I272" s="20" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J272" s="302" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K272" s="20" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L272" s="20" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/bird-f27/branch-current.json;risk-after-ack.json</x:v>
+      </x:c>
+      <x:c r="L272" s="20" t="str">
+        <x:v>R12-MQTT-BIRD-B-703e2e19</x:v>
       </x:c>
     </x:row>
     <x:row r="273" ht="160" customHeight="1">
@@ -41978,19 +42277,19 @@
         <x:v>暂时测不了</x:v>
       </x:c>
       <x:c r="H273" s="20" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：按现有接口提供明确反馈及当前解除依据。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮部分验证，整项未完成：同一鸟类批次已完成发现、风险生成、核验和通知交接，未进无人机研判；配置未启用阻断实际投递，反馈/解除闭环未完成。</x:v>
-      </x:c>
-      <x:c r="I273" s="20" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J273" s="21">
-        <x:v>46293</x:v>
+        <x:v>没有已确认的空间风险解除判据/事实写入接口，不能以停报或签收替代解除；当前依据不足仍保留待确认。</x:v>
+      </x:c>
+      <x:c r="I273" s="20" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J273" s="302" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K273" s="20" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L273" s="20" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/bird-f27/branch-current.json;bird-stop.json</x:v>
+      </x:c>
+      <x:c r="L273" s="20" t="str">
+        <x:v>R12-MQTT-BIRD-B-703e2e19</x:v>
       </x:c>
     </x:row>
     <x:row r="274" ht="160" customHeight="1">
@@ -42016,19 +42315,19 @@
         <x:v>暂时测不了</x:v>
       </x:c>
       <x:c r="H274" s="20" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：核对风险、通知、回执、证据及相关统计。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮部分验证，整项未完成：同一鸟类批次已完成发现、风险生成、核验和通知交接，未进无人机研判；配置未启用阻断实际投递，反馈/解除闭环未完成。</x:v>
-      </x:c>
-      <x:c r="I274" s="20" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J274" s="21">
-        <x:v>46293</x:v>
+        <x:v>风险、核验、通知冻结材料同一组ID；鸟群不进入UAV限定列表。真实解除及对应历史/统计尚缺，完整本步保留未通过。</x:v>
+      </x:c>
+      <x:c r="I274" s="20" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J274" s="302" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K274" s="20" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L274" s="20" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/bird-f27/history-target.json;bird-f27/b-accepted-history.json;fix50-api-counts.json</x:v>
+      </x:c>
+      <x:c r="L274" s="20" t="str">
+        <x:v>R12-MQTT-BIRD-B-703e2e19</x:v>
       </x:c>
     </x:row>
     <x:row r="275" ht="160" customHeight="1">
@@ -42051,22 +42350,22 @@
         <x:v>1439</x:v>
       </x:c>
       <x:c r="G275" s="20" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H275" s="20" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：刷新重登，查历史并结束模拟。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮部分验证，整项未完成：同一鸟类批次已完成发现、风险生成、核验和通知交接，未进无人机研判；配置未启用阻断实际投递，反馈/解除闭环未完成。</x:v>
-      </x:c>
-      <x:c r="I275" s="20" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J275" s="21">
-        <x:v>46293</x:v>
+        <x:v>在重新登录后的5177页面回查同一风险与签收历史，核验1条、通知1条，无重复；原鸟群模拟已停止。</x:v>
+      </x:c>
+      <x:c r="I275" s="20" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J275" s="302" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K275" s="20" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L275" s="20" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/bird-f27/accepted-history-ui.png;bird-stop.json</x:v>
+      </x:c>
+      <x:c r="L275" s="20" t="str">
+        <x:v>R12-MQTT-BIRD-B-703e2e19</x:v>
       </x:c>
     </x:row>
     <x:row r="276" ht="160" customHeight="1">
@@ -43229,22 +43528,22 @@
         <x:v>1532</x:v>
       </x:c>
       <x:c r="G306" s="20" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H306" s="20" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：准备专用测试TCP设备、接入范围、协议版本与账号。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮：未完成整项。缺独立健康GOOD的恢复样本或所需TCP/光电协议测试回执；MQTT在线和UNKNOWN不能冒充健康恢复。</x:v>
-      </x:c>
-      <x:c r="I306" s="20" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J306" s="21">
-        <x:v>46293</x:v>
+        <x:v>独立 PostGIS radar_browser_verify_qa0929r12，回环 TCP58619；仅专用 QA-F31-TCP，simulated=true，live 是协议模式而非现场验收。</x:v>
+      </x:c>
+      <x:c r="I306" s="20" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J306" s="302" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K306" s="20" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L306" s="20" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/radar-f31/onboard-form.txt;scope-fixed-manifest.json</x:v>
+      </x:c>
+      <x:c r="L306" s="20" t="str">
+        <x:v>R12-PG-F31-ce4e5b9b（隔离协议模拟）</x:v>
       </x:c>
     </x:row>
     <x:row r="307" ht="160" customHeight="1">
@@ -43267,22 +43566,22 @@
         <x:v>1535</x:v>
       </x:c>
       <x:c r="G307" s="20" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H307" s="20" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：从统一入口选雷达及支持的TCP协议，保存配置。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮：未完成整项。缺独立健康GOOD的恢复样本或所需TCP/光电协议测试回执；MQTT在线和UNKNOWN不能冒充健康恢复。</x:v>
-      </x:c>
-      <x:c r="I307" s="20" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J307" s="21">
-        <x:v>46293</x:v>
+        <x:v>管理端统一接入页正常保存雷达 TCP3.0.0，固定 ce4e5b9b 设备ID；HOLD 时 OFFLINE/UNKNOWN，保存未冒充在线。</x:v>
+      </x:c>
+      <x:c r="I307" s="20" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J307" s="302" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K307" s="20" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L307" s="20" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/radar-f31/registered-hold.json;onboard-form.txt</x:v>
+      </x:c>
+      <x:c r="L307" s="20" t="str">
+        <x:v>R12-PG-F31-ce4e5b9b（隔离协议模拟）</x:v>
       </x:c>
     </x:row>
     <x:row r="308" ht="160" customHeight="1">
@@ -43305,22 +43604,22 @@
         <x:v>1538</x:v>
       </x:c>
       <x:c r="G308" s="20" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H308" s="20" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：核对型号、单位区域、地址和允许启停状态。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮：未完成整项。缺独立健康GOOD的恢复样本或所需TCP/光电协议测试回执；MQTT在线和UNKNOWN不能冒充健康恢复。</x:v>
-      </x:c>
-      <x:c r="I308" s="20" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J308" s="21">
-        <x:v>46293</x:v>
+        <x:v>实际页面补齐开发测试组织/区域，型号地址不变；标准设备与台账同 ID；范围/字段权限由正式 H2和PG回归验证。</x:v>
+      </x:c>
+      <x:c r="I308" s="20" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J308" s="302" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K308" s="20" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L308" s="20" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/radar-f31/scope-bound.json;scope-bound-ui.png</x:v>
+      </x:c>
+      <x:c r="L308" s="20" t="str">
+        <x:v>R12-PG-F31-ce4e5b9b（隔离协议模拟）</x:v>
       </x:c>
     </x:row>
     <x:row r="309" ht="160" customHeight="1">
@@ -43343,22 +43642,22 @@
         <x:v>1541</x:v>
       </x:c>
       <x:c r="G309" s="20" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H309" s="20" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：创建任务并发起连接。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮：未完成整项。缺独立健康GOOD的恢复样本或所需TCP/光电协议测试回执；MQTT在线和UNKNOWN不能冒充健康恢复。</x:v>
-      </x:c>
-      <x:c r="I309" s="20" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J309" s="21">
-        <x:v>46293</x:v>
+        <x:v>正常页面创建 CT-1790660227643-8AC94F 并连接，保留独立任务ID和受理步骤。</x:v>
+      </x:c>
+      <x:c r="I309" s="20" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J309" s="302" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K309" s="20" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L309" s="20" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/radar-f31/configured-task.txt</x:v>
+      </x:c>
+      <x:c r="L309" s="20" t="str">
+        <x:v>R12-PG-F31-ce4e5b9b（隔离协议模拟）</x:v>
       </x:c>
     </x:row>
     <x:row r="310" ht="160" customHeight="1">
@@ -43381,22 +43680,22 @@
         <x:v>1544</x:v>
       </x:c>
       <x:c r="G310" s="20" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H310" s="20" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：连接成功后保存本次参数，再开始调测。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮：未完成整项。缺独立健康GOOD的恢复样本或所需TCP/光电协议测试回执；MQTT在线和UNKNOWN不能冒充健康恢复。</x:v>
-      </x:c>
-      <x:c r="I310" s="20" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J310" s="21">
-        <x:v>46293</x:v>
+        <x:v>连接后页面保存任务配置，再点击开始协议调测，最终任务版本5。</x:v>
+      </x:c>
+      <x:c r="I310" s="20" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J310" s="302" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K310" s="20" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L310" s="20" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/radar-f31/configured-task.txt;commission-report-before-fix.json</x:v>
+      </x:c>
+      <x:c r="L310" s="20" t="str">
+        <x:v>R12-PG-F31-ce4e5b9b（隔离协议模拟）</x:v>
       </x:c>
     </x:row>
     <x:row r="311" ht="160" customHeight="1">
@@ -43419,22 +43718,22 @@
         <x:v>1547</x:v>
       </x:c>
       <x:c r="G311" s="20" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H311" s="20" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：由模拟器返回真实测试协议响应、心跳和点迹。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮：未完成整项。缺独立健康GOOD的恢复样本或所需TCP/光电协议测试回执；MQTT在线和UNKNOWN不能冒充健康恢复。</x:v>
-      </x:c>
-      <x:c r="I311" s="20" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J311" s="21">
-        <x:v>46293</x:v>
+        <x:v>本机真实 socket 响应登录、心跳、GETREG、RTK及UPLOAD_TRACK_V3；报告分项均有协议依据，无mock适配降级。</x:v>
+      </x:c>
+      <x:c r="I311" s="20" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J311" s="302" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K311" s="20" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L311" s="20" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/radar-f31/commission-report-before-fix.json;scope-fixed-manifest.json</x:v>
+      </x:c>
+      <x:c r="L311" s="20" t="str">
+        <x:v>R12-PG-F31-ce4e5b9b（隔离协议模拟）</x:v>
       </x:c>
     </x:row>
     <x:row r="312" ht="160" customHeight="1">
@@ -43457,22 +43756,22 @@
         <x:v>1550</x:v>
       </x:c>
       <x:c r="G312" s="20" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H312" s="20" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：查看结束状态及完整报告。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮：未完成整项。缺独立健康GOOD的恢复样本或所需TCP/光电协议测试回执；MQTT在线和UNKNOWN不能冒充健康恢复。</x:v>
-      </x:c>
-      <x:c r="I312" s="20" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J312" s="21">
-        <x:v>46293</x:v>
+        <x:v>原报告 PASSED 且 DEVELOPMENT_SIMULATION、confirmed=false；重登后同一任务报告仍可查看，不代表现场验收。</x:v>
+      </x:c>
+      <x:c r="I312" s="20" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J312" s="302" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K312" s="20" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L312" s="20" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/radar-f31/report-relogin.png;commission-report-before-fix.json</x:v>
+      </x:c>
+      <x:c r="L312" s="20" t="str">
+        <x:v>R12-PG-F31-ce4e5b9b（隔离协议模拟）</x:v>
       </x:c>
     </x:row>
     <x:row r="313" ht="160" customHeight="1">
@@ -43495,22 +43794,22 @@
         <x:v>1553</x:v>
       </x:c>
       <x:c r="G313" s="20" t="str">
-        <x:v>暂时测不了</x:v>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="H313" s="20" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：核对设备当前信息、来源时间和健康。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮：未完成整项。缺独立健康GOOD的恢复样本或所需TCP/光电协议测试回执；MQTT在线和UNKNOWN不能冒充健康恢复。</x:v>
-      </x:c>
-      <x:c r="I313" s="20" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J313" s="21">
-        <x:v>46293</x:v>
+        <x:v>实时监测原始航迹31、boot31000000、x/y/z100/200/80、SNR15与报文一致；连续帧更新，位置未派生。</x:v>
+      </x:c>
+      <x:c r="I313" s="20" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J313" s="302" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K313" s="20" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L313" s="20" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/radar-f31/raw-targets-after-fix.json;scope-live-status.json</x:v>
+      </x:c>
+      <x:c r="L313" s="20" t="str">
+        <x:v>R12-PG-F31-ce4e5b9b（隔离协议模拟）</x:v>
       </x:c>
     </x:row>
     <x:row r="314" ht="160" customHeight="1">
@@ -43536,19 +43835,19 @@
         <x:v>暂时测不了</x:v>
       </x:c>
       <x:c r="H314" s="20" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：前台融合感知查本设备原始来源及统一目标。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮：未完成整项。缺独立健康GOOD的恢复样本或所需TCP/光电协议测试回执；MQTT在线和UNKNOWN不能冒充健康恢复。</x:v>
-      </x:c>
-      <x:c r="I314" s="20" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J314" s="21">
-        <x:v>46293</x:v>
+        <x:v>API 已证新统一目标 e34711f8 与本雷达 source QA-F31-TCP、外部31和明确归属一致；前台设备可见。缺少已核验站址/坐标转换依据，目标无WGS84位置，前台不能定位查同一目标；不拿别的目标代替。</x:v>
+      </x:c>
+      <x:c r="I314" s="20" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J314" s="302" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K314" s="20" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L314" s="20" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/radar-f31/unified-scoped-evidence.json;unlocated-device-ui.png</x:v>
+      </x:c>
+      <x:c r="L314" s="20" t="str">
+        <x:v>R12-PG-F31-ce4e5b9b（隔离协议模拟）</x:v>
       </x:c>
     </x:row>
     <x:row r="315" ht="160" customHeight="1">
@@ -43574,19 +43873,19 @@
         <x:v>暂时测不了</x:v>
       </x:c>
       <x:c r="H315" s="20" t="str">
-        <x:v>第十轮：本步尚未作为同一事件完整链路验收。当前步骤：重登回查报告和目标，结束模拟并核对状态变化。。浏览器阻塞已解除；设备回执、角色会话、通知主体/通道、处罚接收方及场景真值是否齐全以本轮报告为准。历史局部证据：第八轮：本流程本步尚未作为同一事件的完整链路验收。第八轮：未完成整项。缺独立健康GOOD的恢复样本或所需TCP/光电协议测试回执；MQTT在线和UNKNOWN不能冒充健康恢复。</x:v>
-      </x:c>
-      <x:c r="I315" s="20" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J315" s="21">
-        <x:v>46293</x:v>
+        <x:v>前后台退出重登成功，原调测报告保留，停报后前台离线且健康未知，最后有效心跳保留，重连不推进时间。统一目标页面回查仍受无可信坐标约束，未完整通过。</x:v>
+      </x:c>
+      <x:c r="I315" s="20" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="J315" s="302" t="n">
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="K315" s="20" t="str">
-        <x:v>第十轮报告；r10-data.json；既有轮次证据</x:v>
-      </x:c>
-      <x:c r="L315" s="20" t="s">
-        <x:v>1216</x:v>
+        <x:v>qa-r12/radar-f31/report-relogin.png;front-offline-ui.png;quiet-device-after.json;qa-r12/radar-f31/offline-heartbeat-preserved.png;heartbeat-fix-offline-retry.json</x:v>
+      </x:c>
+      <x:c r="L315" s="20" t="str">
+        <x:v>R12-PG-F31-ce4e5b9b（隔离协议模拟）</x:v>
       </x:c>
     </x:row>
     <x:row r="316" ht="93" customHeight="1">
@@ -45564,7 +45863,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbce1658c968440b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56fd5ff798ab4d50"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -45616,7 +45915,7 @@
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="17" t="str">
-        <x:v>第十二轮：44处代码缺陷修复并回归；剩余条目含未执行组合与真实外部依赖。旧登录阻塞已解除，详见本轮报告及新增证据。</x:v>
+        <x:v>第十二轮：61处代码缺陷修复并回归；剩余条目含未执行组合与真实外部依赖。旧登录阻塞已解除，详见本轮报告及新增证据。</x:v>
       </x:c>
       <x:c r="B3" s="17"/>
       <x:c r="C3" s="17"/>
@@ -46188,7 +46487,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ff565041827499a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2211270d836a4b10"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -48427,7 +48726,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5fba605b025484b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99ed49199b754b55"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>